<commit_message>
Pin FLUX.1-dev and add the engine watch-list (v0.2.1)
Section 15.5 records Qwen3.8-LiveTranslate (hosted API only, fails
zero-cloud) and Qwen-Image-2.1 (research licence) as considered but not
adopted, with the event that would bring each in. FLUX.1-dev is pinned
as the image engine on quality. Workbook Ref Multimodal sheet follows.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USyWZdFCwDpe3L4dpdaCcG
</commit_message>
<xml_diff>
--- a/docs/ATLAS_BUILD_BASELINE.xlsx
+++ b/docs/ATLAS_BUILD_BASELINE.xlsx
@@ -581,7 +581,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Companion to docs/ATLAS_FRAMEWORK_REVIEW.md v0.2 (2026-09-21). Every decision is closed. Nothing has been executed; the Day 1 script is written against this.</t>
+          <t>Companion to docs/ATLAS_FRAMEWORK_REVIEW.md v0.2.1 (2026-09-21). Every decision is closed. Nothing has been executed; the Day 1 script is written against this.</t>
         </is>
       </c>
     </row>
@@ -1707,14 +1707,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1727,7 +1727,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Section 15. Tools install in Phase 2 (CPU, always available). Engines build in Phase 4 inside ROCm containers.</t>
+          <t>Section 15. Tools install in Phase 2 (CPU, always available). Engines build in Phase 4 inside ROCm containers. The watch-list (15.5) is considered, not adopted.</t>
         </is>
       </c>
     </row>
@@ -1972,12 +1972,12 @@
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>FLUX.1</t>
+          <t>FLUX.1-dev</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Image generation, architectural visualisation with LoRA (the "Arch-DiT" imagery use)</t>
+          <t>Image generation, architectural visualisation with LoRA (the "Arch-DiT" imagery use). The dev variant, chosen for quality over the Apache-licensed schnell variant, the Principal accepts the dev non-commercial licence (15.5)</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
@@ -2425,6 +2425,106 @@
       <c r="E35" s="11" t="inlineStr">
         <is>
           <t>Domains 8 and 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Engine watch-list: considered, not adopted (15.5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>Engine</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>What it does</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>Why not now</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="inlineStr">
+        <is>
+          <t>What would change the answer</t>
+        </is>
+      </c>
+      <c r="E38" s="10" t="inlineStr">
+        <is>
+          <t>Would replace</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>Qwen3.8-LiveTranslate (19 Sep 2026)</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>Real-time simultaneous interpretation: 60 languages understood, 29 spoken, about 2.3 s lag</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>Hosted API only (Alibaba Cloud Model Studio, QwenCloud, WebSocket). No open weights. Fails the zero-cloud rule on inference off-node and audio leaving the machine</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="inlineStr">
+        <is>
+          <t>An open-weights release. Qwen has released weights for Qwen3-Omni, so this is plausible</t>
+        </is>
+      </c>
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>Nothing. Live interpretation is an open gap, the Whisper to engine to Kokoro pipeline does consecutive translation only, in Kokoro's eight languages</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>Qwen-Image-2.1 (20 Sep 2026)</t>
+        </is>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>Image generation and editing in one 7B checkpoint: native RGBA, 2K, up to ten reference images, strongest text-in-image of its class, about 14 GB BF16, GGUF available, plain BF16 path on gfx1151</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>Qwen Research License, non-commercial only. Same restriction that excluded Fish Audio S2 (C20). Not a peer of Qwen2.5-VL-72B, which reads images</t>
+        </is>
+      </c>
+      <c r="D40" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> this one makes them</t>
+        </is>
+      </c>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>Re-licensing to Apache-2.0 (Qwen did this for Qwen2.5 within months) or a commercial licence obtained by the Principal</t>
+        </is>
+      </c>
+      <c r="F40" s="11" t="inlineStr">
+        <is>
+          <t>FLUX.1-dev outright: half the footprint, generate and edit in one model</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Decision recorded 2026-09-21: FLUX.1-dev stays as the image engine, quality being the deciding factor. FLUX.1-dev carries the same non-commercial licence as Qwen-Image-2.1, so the licence does not separate them; validation on gfx1151 does.</t>
         </is>
       </c>
     </row>
@@ -3228,7 +3328,7 @@
       </c>
       <c r="B39" s="11" t="inlineStr">
         <is>
-          <t>2. Build green engines in order of value: FLUX.1, Wan2.2, Florence-2, TimesFM or Chronos, UI-TARS 2.0, Rad-DINO, SAM 2 with the extension flag, Stable Audio Open, CosyVoice2, OpenVLA. The vision engine is not here; Qwen2.5-VL-72B is a GGUF engine pulled in Phase 3.</t>
+          <t>2. Build green engines in order of value: FLUX.1-dev, Wan2.2, Florence-2, TimesFM or Chronos, UI-TARS 2.0, Rad-DINO, SAM 2 with the extension flag, Stable Audio Open, CosyVoice2, OpenVLA. The vision engine is not here; Qwen2.5-VL-72B is a GGUF engine pulled in Phase 3.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix a split cell in the workbook watch-list row
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USyWZdFCwDpe3L4dpdaCcG
</commit_message>
<xml_diff>
--- a/docs/ATLAS_BUILD_BASELINE.xlsx
+++ b/docs/ATLAS_BUILD_BASELINE.xlsx
@@ -1707,7 +1707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2502,20 +2502,15 @@
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Qwen Research License, non-commercial only. Same restriction that excluded Fish Audio S2 (C20). Not a peer of Qwen2.5-VL-72B, which reads images</t>
+          <t>Qwen Research License, non-commercial only. Same restriction that excluded Fish Audio S2 (C20). Not a peer of Qwen2.5-VL-72B, which reads images, this one makes them</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> this one makes them</t>
+          <t>Re-licensing to Apache-2.0 (Qwen did this for Qwen2.5 within months) or a commercial licence obtained by the Principal</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
-        <is>
-          <t>Re-licensing to Apache-2.0 (Qwen did this for Qwen2.5 within months) or a commercial licence obtained by the Principal</t>
-        </is>
-      </c>
-      <c r="F40" s="11" t="inlineStr">
         <is>
           <t>FLUX.1-dev outright: half the footprint, generate and edit in one model</t>
         </is>

</xml_diff>

<commit_message>
Close the build baseline (v0.3): returned workbook complete
Every decision confirmed, all 26 resolutions accepted, all 21 risks
acknowledged and all 16 pre-execution items ticked in the workbook the
Principal returned. Section 22 and the workbook now carry that as the
record; sheet 4 (Verification) is the only open sheet, filled on Day 1.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USyWZdFCwDpe3L4dpdaCcG
</commit_message>
<xml_diff>
--- a/docs/ATLAS_BUILD_BASELINE.xlsx
+++ b/docs/ATLAS_BUILD_BASELINE.xlsx
@@ -581,7 +581,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Companion to docs/ATLAS_FRAMEWORK_REVIEW.md v0.2.1 (2026-09-21). Every decision is closed. Nothing has been executed; the Day 1 script is written against this.</t>
+          <t>Companion to docs/ATLAS_FRAMEWORK_REVIEW.md v0.3 (2026-09-21). Closed baseline: every response given in the workbook returned 2026-09-21. Nothing has been executed; the Day 1 script is written against this.</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>1. Sheet 1 is a closed record: all fourteen decisions, as you answered them. Sheets 2 and 3 are mostly a record too, but eleven rows are blank and need you. Sheet 4 fills during Day 1. Sheet 5 lists the real-world items outstanding.</t>
+          <t>1. Sheets 1, 2, 3 and 5 are a closed record: every decision, resolution, risk and pre-execution item as you answered it on 2026-09-21. Sheet 4 fills during Day 1 and is the only sheet still open.</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>6. What is genuinely outstanding: eleven response cells (six new resolutions on sheet 2, five risk acknowledgements on sheet 3) and four Principal actions on sheet 5 - store the USB recovery drive away from the node, create the Google OAuth client, source the two voice recordings, and have a monitor ready for first boot. The four build-side rows on sheet 5 are yours to tick as the machine is prepared.</t>
+          <t>6. Nothing is outstanding before Day 1. To reopen an item, change its response cell (Changed my mind, Disagree, Discuss or No) and write the reason beside it; the progress table below shows it at once.</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4371,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Section 18. C1 to C20 are already accepted and marked. C21 to C26 are new in v0.2 and blank: please read and answer those six.</t>
+          <t>Section 18. All twenty-six resolutions accepted in the workbook returned 2026-09-21. Closed record; change a cell only to reopen one.</t>
         </is>
       </c>
     </row>
@@ -4878,7 +4878,11 @@
           <t>26.04.1. The 24.04.5 point release backports the same kernel 7.0 and Mesa 26.0, so hardware support is identical; 26.04.1 wins on support life and toolchain (3.1)</t>
         </is>
       </c>
-      <c r="D25" s="16" t="n"/>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>Accept</t>
+        </is>
+      </c>
       <c r="E25" s="17" t="n"/>
     </row>
     <row r="26">
@@ -4897,7 +4901,11 @@
           <t>Neither. The gain is on CPU-bound distribution packages, not GPU inference (3.1)</t>
         </is>
       </c>
-      <c r="D26" s="16" t="n"/>
+      <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>Accept</t>
+        </is>
+      </c>
       <c r="E26" s="17" t="n"/>
     </row>
     <row r="27">
@@ -4916,7 +4924,11 @@
           <t>Q8_0 for Nemotron, Qwen3.5, Qwen2.5-VL-72B and Meditron; MXFP4 retained for gpt-oss as its native form; Q4_K_XL for the Apex engine (5.1)</t>
         </is>
       </c>
-      <c r="D27" s="16" t="n"/>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>Accept</t>
+        </is>
+      </c>
       <c r="E27" s="17" t="n"/>
     </row>
     <row r="28">
@@ -4935,7 +4947,11 @@
           <t>Reserve closed. Six new domains, five subspecialty folds (8.2)</t>
         </is>
       </c>
-      <c r="D28" s="16" t="n"/>
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>Accept</t>
+        </is>
+      </c>
       <c r="E28" s="17" t="n"/>
     </row>
     <row r="29">
@@ -4954,7 +4970,11 @@
           <t>One engine: Qwen2.5-VL-72B at Q8_0. The 32B is real and official, but the Principal chose maximum quality (15.2)</t>
         </is>
       </c>
-      <c r="D29" s="16" t="n"/>
+      <c r="D29" s="16" t="inlineStr">
+        <is>
+          <t>Accept</t>
+        </is>
+      </c>
       <c r="E29" s="17" t="n"/>
     </row>
     <row r="30">
@@ -4973,7 +4993,11 @@
           <t>Two may be resident; exactly one generates, everywhere, including Celery jobs (4.2)</t>
         </is>
       </c>
-      <c r="D30" s="16" t="n"/>
+      <c r="D30" s="16" t="inlineStr">
+        <is>
+          <t>Accept</t>
+        </is>
+      </c>
       <c r="E30" s="17" t="n"/>
     </row>
   </sheetData>
@@ -5023,7 +5047,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Section 20. Already-acknowledged risks are marked. Five rows are blank and need you: R9 and R16 changed wording in v0.2, and R19 to R21 are new.</t>
+          <t>Section 20. All twenty-one risks acknowledged in the workbook returned 2026-09-21. Closed record; change a cell to Discuss only to reopen one.</t>
         </is>
       </c>
     </row>
@@ -5354,7 +5378,11 @@
           <t>The node runs on Wi-Fi by the Principal's choice; V1 is informational</t>
         </is>
       </c>
-      <c r="F13" s="16" t="n"/>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G13" s="17" t="n"/>
     </row>
     <row r="14">
@@ -5383,7 +5411,11 @@
           <t>Own row in the Phase 3 gate; a failure defers the engine without blocking the phase or the other six</t>
         </is>
       </c>
-      <c r="F14" s="16" t="n"/>
+      <c r="F14" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G14" s="17" t="n"/>
     </row>
     <row r="15">
@@ -5412,7 +5444,11 @@
           <t>Phases 3 and 4 detached and resumable; retries are free</t>
         </is>
       </c>
-      <c r="F15" s="16" t="n"/>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G15" s="17" t="n"/>
     </row>
     <row r="16">
@@ -5441,7 +5477,11 @@
           <t>Bound to LAN and WireGuard only, never internet-facing; no desktop autologin</t>
         </is>
       </c>
-      <c r="F16" s="16" t="n"/>
+      <c r="F16" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G16" s="17" t="n"/>
     </row>
     <row r="17">
@@ -5668,7 +5708,11 @@
           <t>Sharpened under D3. The Principal keeps a copy on the node and on an external USB drive. The on-node copy is convenience only; the USB copy is the one that matters, and it must live away from the node, since a fire or burglary that takes the node takes anything beside it. Quarterly restore test</t>
         </is>
       </c>
-      <c r="F23" s="16" t="n"/>
+      <c r="F23" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G23" s="17" t="n"/>
     </row>
     <row r="24">
@@ -6393,7 +6437,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Section 22. Rows already marked Yes are done or automated. Nothing runs until every row reads Yes or N/A.</t>
+          <t>Section 22. Every row ticked in the workbook returned 2026-09-21. Nothing runs until every row reads Yes or N/A; every row does.</t>
         </is>
       </c>
     </row>
@@ -6498,10 +6542,14 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Store the USB recovery drive away from the node, not beside it (R16).</t>
-        </is>
-      </c>
-      <c r="D8" s="16" t="n"/>
+          <t>Store the USB recovery drive away from the node, not beside it (R16). Done.</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="E8" s="17" t="n"/>
     </row>
     <row r="9">
@@ -6515,10 +6563,14 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Create the Google Cloud OAuth client for Gmail, Calendar and Drive, and be reachable for roughly five minutes during the Phase 2 pause (V20). This one step cannot be automated: Google requires the account owner to click Allow.</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="n"/>
+          <t>Create the Google Cloud OAuth client for Gmail, Calendar and Drive, and be reachable for roughly five minutes during the Phase 2 pause (V20). Client created. The consent click itself still happens during Phase 2; Google requires the account owner to click Allow.</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="E9" s="17" t="n"/>
     </row>
     <row r="10">
@@ -6532,10 +6584,14 @@
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Source reference recordings for Alaric's gravelly voice and, if the British male presets collide, Gideon's. Until then both fall back to the nearest Kokoro preset and V7 is recorded as deferred, not failed.</t>
-        </is>
-      </c>
-      <c r="D10" s="16" t="n"/>
+          <t>Source reference recordings for Alaric's gravelly voice and, if the British male presets collide, Gideon's. Sourced. The Day 1 script names the directory they are copied into before Phase 2; if absent, both fall back to the nearest Kokoro preset and V7 is recorded as deferred, not failed.</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="E10" s="17" t="n"/>
     </row>
     <row r="11">
@@ -6549,10 +6605,14 @@
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Have a monitor and keyboard available for Phase 1 only, in case first boot needs a hand.</t>
-        </is>
-      </c>
-      <c r="D11" s="16" t="n"/>
+          <t>Have a monitor and keyboard available for Phase 1 only, in case first boot needs a hand. Done.</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="E11" s="17" t="n"/>
     </row>
     <row r="12">
@@ -6608,10 +6668,14 @@
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Ubuntu Server 26.04.1 installed on the 4 TB drive; 8 TB drive unpartitioned.</t>
-        </is>
-      </c>
-      <c r="D14" s="16" t="n"/>
+          <t>Ubuntu Server 26.04.1 installed on the 4 TB drive; 8 TB drive unpartitioned. Done.</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="E14" s="17" t="n"/>
     </row>
     <row r="15">
@@ -6625,10 +6689,14 @@
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>BIOS: UMA minimum, IOMMU on, fTPM on, Secure Boot disabled (D2).</t>
-        </is>
-      </c>
-      <c r="D15" s="16" t="n"/>
+          <t>BIOS: UMA minimum, IOMMU on, fTPM on, Secure Boot disabled (D2). Done.</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="E15" s="17" t="n"/>
     </row>
     <row r="16">
@@ -6642,10 +6710,14 @@
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>LAN address reserved for the node on the router, over Wi-Fi; UDP 51820 forward confirmed to that address.</t>
-        </is>
-      </c>
-      <c r="D16" s="16" t="n"/>
+          <t>LAN address reserved for the node on the router, over Wi-Fi; UDP 51820 forward confirmed to that address. Done.</t>
+        </is>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="E16" s="17" t="n"/>
     </row>
     <row r="17">
@@ -6659,10 +6731,14 @@
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Internet bandwidth known, so the ~690 GB Phase 3 download can be planned.</t>
-        </is>
-      </c>
-      <c r="D17" s="16" t="n"/>
+          <t>Internet bandwidth known, so the ~690 GB Phase 3 download can be planned. Done; the figure was not recorded in the workbook, so the 100 Mbps planning assumption in 15.4 stands until stated.</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="E17" s="17" t="n"/>
     </row>
     <row r="18">
@@ -6697,10 +6773,14 @@
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>C21 through C26 are new in v0.2 and await an answer on sheet 2 of the workbook: the Ubuntu and amd64v3 rejections, the quantisation rise, the closed reserve list, the vision consolidation, and the residency-versus-generation reading.</t>
-        </is>
-      </c>
-      <c r="D19" s="16" t="n"/>
+          <t>C21 through C26, new in v0.2, accepted in the returned workbook: the Ubuntu and amd64v3 rejections, the quantisation rise, the closed reserve list, the vision consolidation, and the residency-versus-generation reading.</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="E19" s="17" t="n"/>
     </row>
     <row r="20">
@@ -6714,10 +6794,14 @@
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>R9, R16, R19, R20 and R21 await acknowledgement on sheet 3: two changed wording in v0.2, three are new.</t>
-        </is>
-      </c>
-      <c r="D20" s="16" t="n"/>
+          <t>R9, R16, R19, R20 and R21 acknowledged in the returned workbook: two changed wording in v0.2, three were new.</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="E20" s="17" t="n"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Framework review v0.3.1: fold the Day 1 script research corrections into the baseline
New Section 23 lists the 23 corrections (DeepSeek KV ladder and 0731
checkpoint, explicit context-shift and parallel flags, Meditron split
join, run-time checksums, kernel lockup_timeout, TPM PCR 7 binding,
Docker-bridge WireGuard binding and DOCKER-USER egress, AMD gfx1151
wheels, UI-TARS 1.5 and Chronos substitutions, gated FLUX and Stable
Audio licences, sudo-rs). Sections 3.3, 3.4, 4.3, 5.1, 15.2, 15.5, 22
and Appendix B amended in place; Section 17 points to scripts/day1.
Workbook regenerated: two new Section 22 rows for the Principal.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USyWZdFCwDpe3L4dpdaCcG
</commit_message>
<xml_diff>
--- a/docs/ATLAS_BUILD_BASELINE.xlsx
+++ b/docs/ATLAS_BUILD_BASELINE.xlsx
@@ -28,7 +28,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2 Resolutions'!$A$4:$E$30</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3 Risks'!$A$4:$G$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4 Verification'!$A$4:$E$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5 Checklist'!$A$4:$E$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5 Checklist'!$A$4:$E$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -581,7 +581,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Companion to docs/ATLAS_FRAMEWORK_REVIEW.md v0.3 (2026-09-21). Closed baseline: every response given in the workbook returned 2026-09-21. Nothing has been executed; the Day 1 script is written against this.</t>
+          <t>Companion to docs/ATLAS_FRAMEWORK_REVIEW.md v0.3.1 (2026-09-27). Closed baseline with the Day 1 script corrections of Section 23 folded in. Nothing has been executed; the scripts under scripts/day1 are written against this.</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>1. Sheets 1, 2, 3 and 5 are a closed record: every decision, resolution, risk and pre-execution item as you answered it on 2026-09-21. Sheet 4 fills during Day 1 and is the only sheet still open.</t>
+          <t>1. Sheets 1, 2 and 3 are a closed record: every decision, resolution and risk as you answered it on 2026-09-21. Sheet 5 has two new rows from v0.3.1 that need you (the Hugging Face token and licence acceptances; the Cloudflare zone id). Sheet 4 fills during Day 1.</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>6. Nothing is outstanding before Day 1. To reopen an item, change its response cell (Changed my mind, Disagree, Discuss or No) and write the reason beside it; the progress table below shows it at once.</t>
+          <t>6. Outstanding before Day 1: the two new sheet 5 rows. To reopen any other item, change its response cell (Changed my mind, Disagree, Discuss or No) and write the reason beside it; the progress table below shows it at once.</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>COUNTA('5 Checklist'!$A$5:$A$20)</f>
+        <f>COUNTA('5 Checklist'!$A$5:$A$22)</f>
         <v/>
       </c>
       <c r="C25" s="12">
@@ -872,7 +872,7 @@
         <v/>
       </c>
       <c r="D25" s="12">
-        <f>COUNTIF('5 Checklist'!$D$5:$D$20,"Yes")+COUNTIF('5 Checklist'!$D$5:$D$20,"N/A")</f>
+        <f>COUNTIF('5 Checklist'!$D$5:$D$22,"Yes")+COUNTIF('5 Checklist'!$D$5:$D$22,"N/A")</f>
         <v/>
       </c>
       <c r="E25" s="12">
@@ -880,11 +880,11 @@
         <v/>
       </c>
       <c r="F25" s="12">
-        <f>COUNTIF('5 Checklist'!$D$5:$D$20,"No")</f>
+        <f>COUNTIF('5 Checklist'!$D$5:$D$22,"No")</f>
         <v/>
       </c>
       <c r="G25" s="12">
-        <f>COUNTBLANK('5 Checklist'!$D$5:$D$20)</f>
+        <f>COUNTBLANK('5 Checklist'!$D$5:$D$22)</f>
         <v/>
       </c>
     </row>
@@ -1707,7 +1707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>Green, the native florence-community checkpoints, no remote code (Section 23)</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
@@ -2053,17 +2053,17 @@
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>TimesFM or Chronos</t>
+          <t>Chronos (Chronos-Bolt / Chronos-2)</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>Time-series forecasting</t>
+          <t>Time-series forecasting. TimesFM dropped in v0.3.1, its 3.0 release is non-commercial (Section 23)</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>Green, Apache-2.0</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
@@ -2134,12 +2134,12 @@
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>UI-TARS 2.0</t>
+          <t>UI-TARS-1.5-7B</t>
         </is>
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>Vision-driven GUI automation for RewardPay and Wix design</t>
+          <t>Vision-driven GUI automation for RewardPay and Wix design. UI-TARS 2.0 has no open weights (Section 23, watch-list)</t>
         </is>
       </c>
       <c r="C25" s="11" t="inlineStr">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>Verify V8: point-cloud ops often carry custom kernels</t>
+          <t>Verify V8: point-cloud ops often carry custom kernels. Licence CC-BY-NC-4.0, recorded under 16.5</t>
         </is>
       </c>
       <c r="D29" s="11" t="inlineStr">
@@ -2323,7 +2323,7 @@
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>Blender Cycles (HIP)</t>
+          <t>Blender 4.5 LTS, Cycles (HIP)</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
@@ -2465,59 +2465,86 @@
     <row r="39">
       <c r="A39" s="11" t="inlineStr">
         <is>
-          <t>Qwen3.8-LiveTranslate (19 Sep 2026)</t>
+          <t>UI-TARS 2.0</t>
         </is>
       </c>
       <c r="B39" s="11" t="inlineStr">
         <is>
-          <t>Real-time simultaneous interpretation: 60 languages understood, 29 spoken, about 2.3 s lag</t>
+          <t>Vision-driven GUI agent, successor to the 1.5-7B build</t>
         </is>
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>Hosted API only (Alibaba Cloud Model Studio, QwenCloud, WebSocket). No open weights. Fails the zero-cloud rule on inference off-node and audio leaving the machine</t>
+          <t>Technical report only, no open weights as of September 2026</t>
         </is>
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>An open-weights release. Qwen has released weights for Qwen3-Omni, so this is plausible</t>
+          <t>An open-weights release</t>
         </is>
       </c>
       <c r="E39" s="11" t="inlineStr">
         <is>
-          <t>Nothing. Live interpretation is an open gap, the Whisper to engine to Kokoro pipeline does consecutive translation only, in Kokoro's eight languages</t>
+          <t>UI-TARS-1.5-7B</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="11" t="inlineStr">
         <is>
+          <t>Qwen3.8-LiveTranslate (19 Sep 2026)</t>
+        </is>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>Real-time simultaneous interpretation: 60 languages understood, 29 spoken, about 2.3 s lag</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>Hosted API only (Alibaba Cloud Model Studio, QwenCloud, WebSocket). No open weights. Fails the zero-cloud rule on inference off-node and audio leaving the machine</t>
+        </is>
+      </c>
+      <c r="D40" s="11" t="inlineStr">
+        <is>
+          <t>An open-weights release. Qwen has released weights for Qwen3-Omni, so this is plausible</t>
+        </is>
+      </c>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>Nothing. Live interpretation is an open gap, the Whisper to engine to Kokoro pipeline does consecutive translation only, in Kokoro's eight languages</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
           <t>Qwen-Image-2.1 (20 Sep 2026)</t>
         </is>
       </c>
-      <c r="B40" s="11" t="inlineStr">
+      <c r="B41" s="11" t="inlineStr">
         <is>
           <t>Image generation and editing in one 7B checkpoint: native RGBA, 2K, up to ten reference images, strongest text-in-image of its class, about 14 GB BF16, GGUF available, plain BF16 path on gfx1151</t>
         </is>
       </c>
-      <c r="C40" s="11" t="inlineStr">
+      <c r="C41" s="11" t="inlineStr">
         <is>
           <t>Qwen Research License, non-commercial only. Same restriction that excluded Fish Audio S2 (C20). Not a peer of Qwen2.5-VL-72B, which reads images, this one makes them</t>
         </is>
       </c>
-      <c r="D40" s="11" t="inlineStr">
+      <c r="D41" s="11" t="inlineStr">
         <is>
           <t>Re-licensing to Apache-2.0 (Qwen did this for Qwen2.5 within months) or a commercial licence obtained by the Principal</t>
         </is>
       </c>
-      <c r="E40" s="11" t="inlineStr">
+      <c r="E41" s="11" t="inlineStr">
         <is>
           <t>FLUX.1-dev outright: half the footprint, generate and edit in one model</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>Decision recorded 2026-09-21: FLUX.1-dev stays as the image engine, quality being the deciding factor. FLUX.1-dev carries the same non-commercial licence as Qwen-Image-2.1, so the licence does not separate them; validation on gfx1151 does.</t>
         </is>
@@ -6417,7 +6444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6437,7 +6464,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Section 22. Every row ticked in the workbook returned 2026-09-21. Nothing runs until every row reads Yes or N/A; every row does.</t>
+          <t>Section 22. Every original row was ticked in the workbook returned 2026-09-21; two rows are new in v0.3.1 and blank. Nothing runs until every row reads Yes or N/A.</t>
         </is>
       </c>
     </row>
@@ -6563,7 +6590,7 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Create the Google Cloud OAuth client for Gmail, Calendar and Drive, and be reachable for roughly five minutes during the Phase 2 pause (V20). Client created. The consent click itself still happens during Phase 2; Google requires the account owner to click Allow.</t>
+          <t>Create the Google Cloud OAuth client for Gmail, Calendar and Drive, and be reachable for roughly five minutes during the Phase 2 pause (V20). Client created. The consent click itself still happens during Phase 2; Google requires the account owner to click Allow. Drop the client JSON into /srv/atlas/staging/inbox/google-oauth-client.json once Phase 1 has created that folder.</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
@@ -6584,14 +6611,10 @@
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Source reference recordings for Alaric's gravelly voice and, if the British male presets collide, Gideon's. Sourced. The Day 1 script names the directory they are copied into before Phase 2; if absent, both fall back to the nearest Kokoro preset and V7 is recorded as deferred, not failed.</t>
-        </is>
-      </c>
-      <c r="D10" s="16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>New in v0.3.1: create a Hugging Face access token (read scope) and, with the same account, accept the licences of the gated models on huggingface.co: pyannote/speaker-diarization-3.1 and pyannote/segmentation-3.0 (V6), black-forest-labs/FLUX.1-dev and stabilityai/stable-audio-open-1.0 (Phase 4). Phase 2 asks for the token once at its start and stores it under /etc/atlas/secrets/; a 403 during a pull names the licence page to visit.</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="n"/>
       <c r="E10" s="17" t="n"/>
     </row>
     <row r="11">
@@ -6605,14 +6628,10 @@
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Have a monitor and keyboard available for Phase 1 only, in case first boot needs a hand. Done.</t>
-        </is>
-      </c>
-      <c r="D11" s="16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>New in v0.3.1: have the Cloudflare zone id for sovereign-node.link to hand (Overview page of the zone). A Zone:DNS:Edit-only token cannot look the zone up by name; Phase 1 step 7 asks for the id once if the token cannot list zones.</t>
+        </is>
+      </c>
+      <c r="D11" s="16" t="n"/>
       <c r="E11" s="17" t="n"/>
     </row>
     <row r="12">
@@ -6621,12 +6640,12 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Automated on the Principal's instruction, no action needed</t>
+          <t>Principal's actions — what is genuinely left</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Cloudflare token relocation and deletion of CLOUDFLARE.txt: Phase 2 step 6b (V23).</t>
+          <t>Source reference recordings for Alaric's gravelly voice and, if the British male presets collide, Gideon's. Sourced. The Day 1 script names the directory they are copied into before Phase 2; if absent, both fall back to the nearest Kokoro preset and V7 is recorded as deferred, not failed.</t>
         </is>
       </c>
       <c r="D12" s="16" t="inlineStr">
@@ -6642,12 +6661,12 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Automated on the Principal's instruction, no action needed</t>
+          <t>Principal's actions — what is genuinely left</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Director aliases generated from names rather than confirmed one by one (D14).</t>
+          <t>Have a monitor and keyboard available for Phase 1 only, in case first boot needs a hand. Done.</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr">
@@ -6663,12 +6682,12 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Build-side preconditions</t>
+          <t>Automated on the Principal's instruction, no action needed</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Ubuntu Server 26.04.1 installed on the 4 TB drive; 8 TB drive unpartitioned. Done.</t>
+          <t>Cloudflare token relocation and deletion of CLOUDFLARE.txt: Phase 2 step 6b (V23).</t>
         </is>
       </c>
       <c r="D14" s="16" t="inlineStr">
@@ -6684,12 +6703,12 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Build-side preconditions</t>
+          <t>Automated on the Principal's instruction, no action needed</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>BIOS: UMA minimum, IOMMU on, fTPM on, Secure Boot disabled (D2). Done.</t>
+          <t>Director aliases generated from names rather than confirmed one by one (D14).</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr">
@@ -6710,7 +6729,7 @@
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>LAN address reserved for the node on the router, over Wi-Fi; UDP 51820 forward confirmed to that address. Done.</t>
+          <t>Ubuntu Server 26.04.1 installed on the 4 TB drive; 8 TB drive unpartitioned. Done.</t>
         </is>
       </c>
       <c r="D16" s="16" t="inlineStr">
@@ -6731,7 +6750,7 @@
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Internet bandwidth known, so the ~690 GB Phase 3 download can be planned. Done; the figure was not recorded in the workbook, so the 100 Mbps planning assumption in 15.4 stands until stated.</t>
+          <t>BIOS: UMA minimum, IOMMU on, fTPM on, Secure Boot disabled (D2). Done.</t>
         </is>
       </c>
       <c r="D17" s="16" t="inlineStr">
@@ -6747,12 +6766,12 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Accepted resolutions</t>
+          <t>Build-side preconditions</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>C1 through C20 accepted in the returned workbook. C19 was reopened and re-decided in the Principal's favour.</t>
+          <t>LAN address reserved for the node on the router, over Wi-Fi; UDP 51820 forward confirmed to that address. Done.</t>
         </is>
       </c>
       <c r="D18" s="16" t="inlineStr">
@@ -6768,12 +6787,12 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Accepted resolutions</t>
+          <t>Build-side preconditions</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>C21 through C26, new in v0.2, accepted in the returned workbook: the Ubuntu and amd64v3 rejections, the quantisation rise, the closed reserve list, the vision consolidation, and the residency-versus-generation reading.</t>
+          <t>Internet bandwidth known, so the ~690 GB Phase 3 download can be planned. Done; the figure was not recorded in the workbook, so the 100 Mbps planning assumption in 15.4 stands until stated.</t>
         </is>
       </c>
       <c r="D19" s="16" t="inlineStr">
@@ -6794,19 +6813,61 @@
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
+          <t>C1 through C20 accepted in the returned workbook. C19 was reopened and re-decided in the Principal's favour.</t>
+        </is>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Accepted resolutions</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>C21 through C26, new in v0.2, accepted in the returned workbook: the Ubuntu and amd64v3 rejections, the quantisation rise, the closed reserve list, the vision consolidation, and the residency-versus-generation reading.</t>
+        </is>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E21" s="17" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Accepted resolutions</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
           <t>R9, R16, R19, R20 and R21 acknowledged in the returned workbook: two changed wording in v0.2, three were new.</t>
         </is>
       </c>
-      <c r="D20" s="16" t="inlineStr">
+      <c r="D22" s="16" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E20" s="17" t="n"/>
+      <c r="E22" s="17" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E20"/>
-  <conditionalFormatting sqref="D5:D20">
+  <autoFilter ref="A4:E22"/>
+  <conditionalFormatting sqref="D5:D22">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Yes"</formula>
     </cfRule>
@@ -6818,7 +6879,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="D5:D20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Choose" prompt="Pick one: Yes / No / N/A" type="list" errorStyle="stop">
+    <dataValidation sqref="D5:D22" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Choose" prompt="Pick one: Yes / No / N/A" type="list" errorStyle="stop">
       <formula1>"Yes,No,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6941,7 +7002,7 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>MXFP4, native</t>
+          <t>MXFP4, re-quantised (Section 23: the abliteration is applied to the BF16 upcast; the MXFP4 GGUF is a requant, same size and speed, the "no accuracy cost" argument below does not transfer)</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
@@ -6968,7 +7029,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>120B hybrid Mamba MoE, 12.7B active</t>
+          <t>120B hybrid Mamba MoE, 12B active (A12B)</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
@@ -7027,7 +7088,7 @@
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
         <is>
-          <t>DeepSeek V4 Flash</t>
+          <t>DeepSeek V4 Flash (0731 checkpoint, MIT)</t>
         </is>
       </c>
       <c r="B10" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Framework review v0.3.2: Day 1 scripts delivered; D15 reopened, R22/R23, Section 17 steps 6d and 9b, Section 22 additions
Section 23 S24-S28 record what the build had to add (sandbox and vault
steps, a second sudoers fragment, the Docker-group risk) and what is Day 2
(send channels, TLS for the app install). D15 puts the Secure Boot versus
TPM-binding choice to the Principal with a recommendation. Section 22
gains the SSH key, encrypted-LVM, atlas.env CONFIRM keys, smb.cred,
Desktop-app OAuth client and USB close-out items. Workbook regenerated:
D15, R22, R23 and the new sheet 5 rows are blank for the Principal.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USyWZdFCwDpe3L4dpdaCcG
</commit_message>
<xml_diff>
--- a/docs/ATLAS_BUILD_BASELINE.xlsx
+++ b/docs/ATLAS_BUILD_BASELINE.xlsx
@@ -24,11 +24,11 @@
     <sheet name="Ref Hardware" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1 Decisions'!$A$4:$F$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1 Decisions'!$A$4:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2 Resolutions'!$A$4:$E$30</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3 Risks'!$A$4:$G$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3 Risks'!$A$4:$G$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4 Verification'!$A$4:$E$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5 Checklist'!$A$4:$E$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5 Checklist'!$A$4:$E$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -581,7 +581,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Companion to docs/ATLAS_FRAMEWORK_REVIEW.md v0.3.1 (2026-09-27). Closed baseline with the Day 1 script corrections of Section 23 folded in. Nothing has been executed; the scripts under scripts/day1 are written against this.</t>
+          <t>Companion to docs/ATLAS_FRAMEWORK_REVIEW.md v0.3.2 (2026-10-04). The Day 1 scripts are delivered under scripts/day1; this workbook carries what the Principal must still answer before running them. Nothing has been executed.</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>1. Sheets 1, 2 and 3 are a closed record: every decision, resolution and risk as you answered it on 2026-09-21. Sheet 5 has two new rows from v0.3.1 that need you (the Hugging Face token and licence acceptances; the Cloudflare zone id). Sheet 4 fills during Day 1.</t>
+          <t>1. Sheets 1, 2 and 3 are a record of your answers of 2026-09-21, with three new rows that need you: D15 on sheet 1 (Secure Boot and the TPM binding), R22 and R23 on sheet 3. Sheet 5 has the pre-execution rows new in v0.3.1 and v0.3.2. Sheet 4 fills during Day 1.</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>6. Outstanding before Day 1: the two new sheet 5 rows. To reopen any other item, change its response cell (Changed my mind, Disagree, Discuss or No) and write the reason beside it; the progress table below shows it at once.</t>
+          <t>6. Outstanding before Day 1: D15, R22, R23 and the blank sheet 5 rows. To reopen any other item, change its response cell (Changed my mind, Disagree, Discuss or No) and write the reason beside it; the progress table below shows it at once.</t>
         </is>
       </c>
     </row>
@@ -740,7 +740,7 @@
         </is>
       </c>
       <c r="B21" s="12">
-        <f>COUNTA('1 Decisions'!$A$5:$A$18)</f>
+        <f>COUNTA('1 Decisions'!$A$5:$A$19)</f>
         <v/>
       </c>
       <c r="C21" s="12">
@@ -748,7 +748,7 @@
         <v/>
       </c>
       <c r="D21" s="12">
-        <f>COUNTIF('1 Decisions'!$E$5:$E$18,"Confirmed")</f>
+        <f>COUNTIF('1 Decisions'!$E$5:$E$19,"Confirmed")</f>
         <v/>
       </c>
       <c r="E21" s="12">
@@ -756,11 +756,11 @@
         <v/>
       </c>
       <c r="F21" s="12">
-        <f>COUNTIF('1 Decisions'!$E$5:$E$18,"Changed my mind")</f>
+        <f>COUNTIF('1 Decisions'!$E$5:$E$19,"Changed my mind")</f>
         <v/>
       </c>
       <c r="G21" s="12">
-        <f>COUNTBLANK('1 Decisions'!$E$5:$E$18)</f>
+        <f>COUNTBLANK('1 Decisions'!$E$5:$E$19)</f>
         <v/>
       </c>
     </row>
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="B23" s="12">
-        <f>COUNTA('3 Risks'!$A$5:$A$25)</f>
+        <f>COUNTA('3 Risks'!$A$5:$A$27)</f>
         <v/>
       </c>
       <c r="C23" s="12">
@@ -810,7 +810,7 @@
         <v/>
       </c>
       <c r="D23" s="12">
-        <f>COUNTIF('3 Risks'!$F$5:$F$25,"Yes")</f>
+        <f>COUNTIF('3 Risks'!$F$5:$F$27,"Yes")</f>
         <v/>
       </c>
       <c r="E23" s="12">
@@ -818,11 +818,11 @@
         <v/>
       </c>
       <c r="F23" s="12">
-        <f>COUNTIF('3 Risks'!$F$5:$F$25,"Discuss")</f>
+        <f>COUNTIF('3 Risks'!$F$5:$F$27,"Discuss")</f>
         <v/>
       </c>
       <c r="G23" s="12">
-        <f>COUNTBLANK('3 Risks'!$F$5:$F$25)</f>
+        <f>COUNTBLANK('3 Risks'!$F$5:$F$27)</f>
         <v/>
       </c>
     </row>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>COUNTA('5 Checklist'!$A$5:$A$22)</f>
+        <f>COUNTA('5 Checklist'!$A$5:$A$26)</f>
         <v/>
       </c>
       <c r="C25" s="12">
@@ -872,7 +872,7 @@
         <v/>
       </c>
       <c r="D25" s="12">
-        <f>COUNTIF('5 Checklist'!$D$5:$D$22,"Yes")+COUNTIF('5 Checklist'!$D$5:$D$22,"N/A")</f>
+        <f>COUNTIF('5 Checklist'!$D$5:$D$26,"Yes")+COUNTIF('5 Checklist'!$D$5:$D$26,"N/A")</f>
         <v/>
       </c>
       <c r="E25" s="12">
@@ -880,11 +880,11 @@
         <v/>
       </c>
       <c r="F25" s="12">
-        <f>COUNTIF('5 Checklist'!$D$5:$D$22,"No")</f>
+        <f>COUNTIF('5 Checklist'!$D$5:$D$26,"No")</f>
         <v/>
       </c>
       <c r="G25" s="12">
-        <f>COUNTBLANK('5 Checklist'!$D$5:$D$22)</f>
+        <f>COUNTBLANK('5 Checklist'!$D$5:$D$26)</f>
         <v/>
       </c>
     </row>
@@ -2923,7 +2923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B43"/>
+  <dimension ref="A1:B45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3242,7 +3242,7 @@
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>7. restic repository on the second drive; nightly timer; first backup; first restore test.</t>
+          <t>6d. AEGIS sandbox image (Section 16.4): built and proved by killing a runaway process under the memory cap (V17). *Added in v0.3.2; the build showed Section 17 had no home for V17.*</t>
         </is>
       </c>
     </row>
@@ -3254,7 +3254,7 @@
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>8. Sentinel timer, enabled with the feeds closed under D6: CoinDesk, an ASX and US index feed, RSS news, node telemetry. Pruning timer.</t>
+          <t>7. restic repository on the second drive; nightly timer; first backup; first restore test.</t>
         </is>
       </c>
     </row>
@@ -3266,7 +3266,7 @@
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>9. Windows PC share mount unit, on-demand.</t>
+          <t>8. Sentinel timer, enabled with the feeds closed under D6: CoinDesk, an ASX and US index feed, RSS news, node telemetry. Pruning timer.</t>
         </is>
       </c>
     </row>
@@ -3278,31 +3278,31 @@
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>10. Gate: every service healthy; V3 second half (llama-cli --list-devices reports ~170 GB), V6, V7 (listening test, deferred if the reference recordings do not exist yet), V12, V20, V23 recorded. The Arbiter's refusal logic is unit-tested here against stub footprints; the real two-engine test is V21 in Phase 3.</t>
+          <t>9. Windows PC share mount unit, on-demand.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>Phase 3</t>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>1. Pull, with checksum verification, at the quantisations fixed in Section 5.1: gpt-oss-120b (MXFP4), gpt-oss-120b abliterated (MXFP4), Nemotron 3 Super (Q8_0), Qwen3.5-122B-A10B (Q8_0), DeepSeek V4 Flash (UD-Q4_K_XL), Qwen2.5-VL-72B (Q8_0), Meditron-70B (Q8_0). About 690 GB.</t>
+          <t>9b. Vault (Section 11): gocryptfs initialised with a passphrase the Principal types once, the open/lock/idle mechanics proved, and the memory rule proved (V18). *Added in v0.3.2.*</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
         <is>
-          <t>Phase 3</t>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
-          <t>2. For each model, in turn: load through the Engine Arbiter; confirm the quantised KV cache actually applied (V4); measure decode and prefill at 512 and 8k tokens; measure swap time; unload; confirm memory returned.</t>
+          <t>10. Gate: every service healthy; V3 second half (llama-cli --list-devices reports ~170 GB), V6, V7 (listening test, deferred if the reference recordings do not exist yet), V12, V13, V14 first half, V15, V16, V17, V18, V20, V23 recorded, plus V10's resident-router half. The Arbiter's refusal logic is unit-tested here against stub footprints; the real two-engine test is V21 in Phase 3. Tool installs whose inputs could not be verified in advance (Bonsai, Blender, OpenStudio/EnergyPlus, MCP4IFC, the build container) record a deferred T-&lt;tool&gt; row and never block the gate; --force 06 re-runs them.</t>
         </is>
       </c>
     </row>
@@ -3314,7 +3314,7 @@
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>3. Two-residency test: load gpt-oss-120b and Qwen2.5-VL-72B together, confirm both hold at ~142 GB, and confirm a second generation request queues rather than running concurrently (V14, V21).</t>
+          <t>1. Pull, with checksum verification, at the quantisations fixed in Section 5.1: gpt-oss-120b (MXFP4), gpt-oss-120b abliterated (MXFP4), Nemotron 3 Super (Q8_0), Qwen3.5-122B-A10B (Q8_0), DeepSeek V4 Flash (UD-Q4_K_XL), Qwen2.5-VL-72B (Q8_0), Meditron-70B (Q8_0). About 690 GB.</t>
         </is>
       </c>
     </row>
@@ -3326,31 +3326,31 @@
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>4. Gate: printed table of load success, KV type, tok/s, swap seconds per engine. This is the day-one load test the whole design depends on (V10). DeepSeek V4 Flash carries its own row: mainline llama.cpp support for this architecture is newer than the rest, so a failure here downgrades it to deferred without blocking the phase (R19).</t>
+          <t>2. For each model, in turn: load through the Engine Arbiter; confirm the quantised KV cache actually applied (V4); measure decode and prefill at 512 and 8k tokens; measure swap time; unload; confirm memory returned.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Phase 3</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>1. Inside the base ROCm container, confirm rocminfo reports gfx1151, then self-test the community PyTorch wheel: tensor on GPU, matmul, a small diffusion step (V11). This is the first and only place ROCm runs.</t>
+          <t>3. Two-residency test: load gpt-oss-120b and Qwen2.5-VL-72B together, confirm both hold at ~142 GB, and confirm a second generation request queues rather than running concurrently (V14, V21).</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="11" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Phase 3</t>
         </is>
       </c>
       <c r="B39" s="11" t="inlineStr">
         <is>
-          <t>2. Build green engines in order of value: FLUX.1-dev, Wan2.2, Florence-2, TimesFM or Chronos, UI-TARS 2.0, Rad-DINO, SAM 2 with the extension flag, Stable Audio Open, CosyVoice2, OpenVLA. The vision engine is not here; Qwen2.5-VL-72B is a GGUF engine pulled in Phase 3.</t>
+          <t>4. Gate: printed table of load success, KV type, tok/s, swap seconds per engine. This is the day-one load test the whole design depends on (V10). DeepSeek V4 Flash carries its own row: mainline llama.cpp support for this architecture is newer than the rest, so a failure here downgrades it to deferred without blocking the phase (R19).</t>
         </is>
       </c>
     </row>
@@ -3362,7 +3362,7 @@
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>3. Attempt yellow engines: TRELLIS, Blender Cycles HIP with CPU fallback. Log pass or fail, never block.</t>
+          <t>1. Inside the base ROCm container, confirm rocminfo reports gfx1151, then self-test the community PyTorch wheel: tensor on GPU, matmul, a small diffusion step (V11). This is the first and only place ROCm runs.</t>
         </is>
       </c>
     </row>
@@ -3374,7 +3374,7 @@
       </c>
       <c r="B41" s="11" t="inlineStr">
         <is>
-          <t>4. Verify PointLLM (V8) and Clay or Prithvi (V9); mark deferred if they fail.</t>
+          <t>2. Build green engines in order of value: FLUX.1-dev, Wan2.2, Florence-2, TimesFM or Chronos, UI-TARS 2.0, Rad-DINO, SAM 2 with the extension flag, Stable Audio Open, CosyVoice2, OpenVLA. The vision engine is not here; Qwen2.5-VL-72B is a GGUF engine pulled in Phase 3.</t>
         </is>
       </c>
     </row>
@@ -3386,7 +3386,7 @@
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>5. Register every passing engine with the Engine Arbiter with its measured footprint.</t>
+          <t>3. Attempt yellow engines: TRELLIS, Blender Cycles HIP with CPU fallback. Log pass or fail, never block.</t>
         </is>
       </c>
     </row>
@@ -3397,6 +3397,30 @@
         </is>
       </c>
       <c r="B43" s="11" t="inlineStr">
+        <is>
+          <t>4. Verify PointLLM (V8) and Clay or Prithvi (V9); mark deferred if they fail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="11" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B44" s="11" t="inlineStr">
+        <is>
+          <t>5. Register every passing engine with the Engine Arbiter with its measured footprint.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="11" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B45" s="11" t="inlineStr">
         <is>
           <t>6. Gate: per-engine table: built, loaded, sample output produced, footprint, pass/fail/deferred.</t>
         </is>
@@ -3904,7 +3928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3925,7 +3949,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Section 19. All fourteen are closed. This sheet is a record: change a row only if you have changed your mind since the workbook was returned.</t>
+          <t>Section 19. Fourteen are closed; D15 (Secure Boot and the TPM binding) is open and needs your answer in the response column, with the option letter in the next column.</t>
         </is>
       </c>
     </row>
@@ -4353,9 +4377,33 @@
       </c>
       <c r="F18" s="17" t="n"/>
     </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>D15</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Secure Boot and the TPM binding (reopens D2)</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>OPEN. D2 disables Secure Boot; S9 binds the TPM2 unlock to PCR 7. With Secure Boot off, PCR 7 is the same for any boot medium, so the data volume unseals for any OS booted on this hardware: the encryption then protects against disk removal, not theft of the whole node. Pre-flight stops until the Principal chooses. Options: (a) enable Secure Boot in the BIOS and keep PCR 7 — reverses D2, but this stack has no out-of-tree kernel modules (amdgpu and WireGuard are in-tree, Docker needs none), so the module-signing friction D2 feared does not arise, and no script change is needed; (b) keep Secure Boot off and bind PCRs 0+4+7 (firmware and boot-loader measurements), which also defeats foreign boot media, at the cost of a re-enrolment with the recovery key after a firmware or GRUB update — a one-line change to the Phase 1 script; (c) keep Secure Boot off and accept the weaker binding by writing ATLAS_ACCEPT_PCR7_NO_SB=1 in /etc/atlas/atlas.env, recorded on every V2 row</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>Recommendation: (a). Awaiting the Principal; the workbook carries the row</t>
+        </is>
+      </c>
+      <c r="E19" s="16" t="n"/>
+      <c r="F19" s="17" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:F18"/>
-  <conditionalFormatting sqref="E5:E18">
+  <autoFilter ref="A4:F19"/>
+  <conditionalFormatting sqref="E5:E19">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Confirmed"</formula>
     </cfRule>
@@ -4364,7 +4412,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="E5:E18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Choose" prompt="Pick one: Confirmed / Changed my mind" type="list" errorStyle="stop">
+    <dataValidation sqref="E5:E19" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Choose" prompt="Pick one: Confirmed / Changed my mind" type="list" errorStyle="stop">
       <formula1>"Confirmed,Changed my mind"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5052,7 +5100,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5074,7 +5122,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Section 20. All twenty-one risks acknowledged in the workbook returned 2026-09-21. Closed record; change a cell to Discuss only to reopen one.</t>
+          <t>Section 20. R1 to R21 acknowledged in the workbook returned 2026-09-21. R22 and R23 are new in v0.3.2 and blank.</t>
         </is>
       </c>
     </row>
@@ -5514,12 +5562,12 @@
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>R10</t>
+          <t>R22</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Sustained thermal load in a small chassis</t>
+          <t>The atlas service user is in the docker group, which is root-equivalent on the host; the orchestrator needs the socket for the sandbox and Phase 4 containers</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
@@ -5529,63 +5577,55 @@
       </c>
       <c r="D17" s="11" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High if the orchestrator is ever compromised</t>
         </is>
       </c>
       <c r="E17" s="11" t="inlineStr">
         <is>
-          <t>Monitor temperatures in Cockpit; the chip's configurable ceiling is 120 W and the Principal is adding external cooling</t>
-        </is>
-      </c>
-      <c r="F17" s="16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>Accepted for Day 1 and recorded in every script header; Day 2 options are rootless Docker or a socket proxy that allows only the sandbox and engine images. New in v0.3.2</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="n"/>
       <c r="G17" s="17" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>R11</t>
+          <t>R23</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>CGNAT prevents inbound WireGuard</t>
+          <t>TPM2 unlock bound to PCR 7 with Secure Boot disabled unseals for any boot medium (see D15)</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Low, port forward already succeeded</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>High for remote access</t>
+          <t>High for physical theft of the node</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>V5 from mobile data, static IP from the ISP if needed</t>
-        </is>
-      </c>
-      <c r="F18" s="16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>Decision D15; until it is made, Phase 1 pre-flight refuses to enrol. New in v0.3.2</t>
+        </is>
+      </c>
+      <c r="F18" s="16" t="n"/>
       <c r="G18" s="17" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>R12</t>
+          <t>R10</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Fictitious directors corresponding as humans, AI non-disclosure</t>
+          <t>Sustained thermal load in a small chassis</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
@@ -5595,12 +5635,12 @@
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>Medium to high, legal</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>Gideon's sensitive-tier check, approval gate, 16.5</t>
+          <t>Monitor temperatures in Cockpit; the chip's configurable ceiling is 120 W and the Principal is adding external cooling</t>
         </is>
       </c>
       <c r="F19" s="16" t="inlineStr">
@@ -5613,27 +5653,27 @@
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
         <is>
-          <t>R13</t>
+          <t>R11</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Abliterated engine used for external output</t>
+          <t>CGNAT prevents inbound WireGuard</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low, port forward already succeeded</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High for remote access</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>Abliterated output always passes the same gate, never routine tier</t>
+          <t>V5 from mobile data, static IP from the ISP if needed</t>
         </is>
       </c>
       <c r="F20" s="16" t="inlineStr">
@@ -5646,12 +5686,12 @@
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>R14</t>
+          <t>R12</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>Chatterbox continuation quirk in production speech</t>
+          <t>Fictitious directors corresponding as humans, AI non-disclosure</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
@@ -5661,12 +5701,12 @@
       </c>
       <c r="D21" s="11" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium to high, legal</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
         <is>
-          <t>V7 testing, Kokoro fallback per line</t>
+          <t>Gideon's sensitive-tier check, approval gate, 16.5</t>
         </is>
       </c>
       <c r="F21" s="16" t="inlineStr">
@@ -5679,27 +5719,27 @@
     <row r="22">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>R15</t>
+          <t>R13</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>Prompt bloat from domain injection makes every dispatch slow</t>
+          <t>Abliterated engine used for external output</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>High without limits</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>High, usability</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>Three-card limit, compact cards, stable-prefix ordering (8.4, 4.4)</t>
+          <t>Abliterated output always passes the same gate, never routine tier</t>
         </is>
       </c>
       <c r="F22" s="16" t="inlineStr">
@@ -5712,27 +5752,27 @@
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>R16</t>
+          <t>R14</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>Backup passphrase or LUKS key lost with the node</t>
+          <t>Chatterbox continuation quirk in production speech</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="D23" s="11" t="inlineStr">
-        <is>
-          <t>Catastrophic</t>
-        </is>
-      </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>Sharpened under D3. The Principal keeps a copy on the node and on an external USB drive. The on-node copy is convenience only; the USB copy is the one that matters, and it must live away from the node, since a fire or burglary that takes the node takes anything beside it. Quarterly restore test</t>
+          <t>V7 testing, Kokoro fallback per line</t>
         </is>
       </c>
       <c r="F23" s="16" t="inlineStr">
@@ -5745,27 +5785,27 @@
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>R17</t>
+          <t>R15</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>PyAnnote gated model not accepted, diarisation silently absent</t>
+          <t>Prompt bloat from domain injection makes every dispatch slow</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High without limits</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High, usability</t>
         </is>
       </c>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>V6</t>
+          <t>Three-card limit, compact cards, stable-prefix ordering (8.4, 4.4)</t>
         </is>
       </c>
       <c r="F24" s="16" t="inlineStr">
@@ -5778,39 +5818,105 @@
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
+          <t>R16</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Backup passphrase or LUKS key lost with the node</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>Catastrophic</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
+          <t>Sharpened under D3. The Principal keeps a copy on the node and on an external USB drive. The on-node copy is convenience only; the USB copy is the one that matters, and it must live away from the node, since a fire or burglary that takes the node takes anything beside it. Quarterly restore test</t>
+        </is>
+      </c>
+      <c r="F25" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G25" s="17" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>R17</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>PyAnnote gated model not accepted, diarisation silently absent</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>V6</t>
+        </is>
+      </c>
+      <c r="F26" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G26" s="17" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
           <t>R18</t>
         </is>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>Continuous vision enabled by drift rather than decision</t>
         </is>
       </c>
-      <c r="C25" s="11" t="inlineStr">
+      <c r="C27" s="11" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="D25" s="11" t="inlineStr">
+      <c r="D27" s="11" t="inlineStr">
         <is>
           <t>High, privacy</t>
         </is>
       </c>
-      <c r="E25" s="11" t="inlineStr">
+      <c r="E27" s="11" t="inlineStr">
         <is>
           <t>Separate capability flag under Alaric, logged, D8 item 7</t>
         </is>
       </c>
-      <c r="F25" s="16" t="inlineStr">
+      <c r="F27" s="16" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G25" s="17" t="n"/>
+      <c r="G27" s="17" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G25"/>
-  <conditionalFormatting sqref="F5:F25">
+  <autoFilter ref="A4:G27"/>
+  <conditionalFormatting sqref="F5:F27">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Yes"</formula>
     </cfRule>
@@ -5819,7 +5925,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F5:F25" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Choose" prompt="Pick one: Yes / Discuss" type="list" errorStyle="stop">
+    <dataValidation sqref="F5:F27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Choose" prompt="Pick one: Yes / Discuss" type="list" errorStyle="stop">
       <formula1>"Yes,Discuss"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6444,7 +6550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6464,7 +6570,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Section 22. Every original row was ticked in the workbook returned 2026-09-21; two rows are new in v0.3.1 and blank. Nothing runs until every row reads Yes or N/A.</t>
+          <t>Section 22. The original rows were ticked in the workbook returned 2026-09-21; the rows new in v0.3.1 and v0.3.2 are blank. Nothing runs until every row reads Yes or N/A.</t>
         </is>
       </c>
     </row>
@@ -6569,14 +6675,10 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Store the USB recovery drive away from the node, not beside it (R16). Done.</t>
-        </is>
-      </c>
-      <c r="D8" s="16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>Have the USB recovery drive present on Day 1 and write it at the Day 1 close-out: the LUKS recovery key (shown once in Phase 1 step 2), the restic passphrase (/etc/atlas/secrets/restic.pass, shown once in Phase 2 step 7) and the vault passphrase you chose (step 9b); then store it away from the node, not beside it (R16). *Reworded in v0.3.2: the material does not exist before Day 1, so the drive cannot be "stored" yet.*</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="n"/>
       <c r="E8" s="17" t="n"/>
     </row>
     <row r="9">
@@ -6590,14 +6692,10 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Create the Google Cloud OAuth client for Gmail, Calendar and Drive, and be reachable for roughly five minutes during the Phase 2 pause (V20). Client created. The consent click itself still happens during Phase 2; Google requires the account owner to click Allow. Drop the client JSON into /srv/atlas/staging/inbox/google-oauth-client.json once Phase 1 has created that folder.</t>
-        </is>
-      </c>
-      <c r="D9" s="16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>New in v0.3.2: your SSH public key in ~/.ssh/authorized_keys on the node before Phase 1 (step 4 turns password login off; pre-flight stops if the file is missing).</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="n"/>
       <c r="E9" s="17" t="n"/>
     </row>
     <row r="10">
@@ -6611,7 +6709,7 @@
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>New in v0.3.1: create a Hugging Face access token (read scope) and, with the same account, accept the licences of the gated models on huggingface.co: pyannote/speaker-diarization-3.1 and pyannote/segmentation-3.0 (V6), black-forest-labs/FLUX.1-dev and stabilityai/stable-audio-open-1.0 (Phase 4). Phase 2 asks for the token once at its start and stores it under /etc/atlas/secrets/; a 403 during a pull names the licence page to visit.</t>
+          <t>New in v0.3.2: fill the CONFIRM keys in /etc/atlas/atlas.env when the first run installs it: GOOGLE_ACCOUNTS (two addresses, each tagged corporate or estate), WINDOWS_SHARE (//host/share), FAMILY_NAMES (for the router's hard rule), BUILDFARM_ACCEPT_ANDROID_SDK_LICENCE (Google's Android SDK licence, needed by the build container), and ATLAS_ACCEPT_PCR7_NO_SB only if D15 is decided as option (c). The first run prints every blank key with an example value and stops.</t>
         </is>
       </c>
       <c r="D10" s="16" t="n"/>
@@ -6628,7 +6726,7 @@
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>New in v0.3.1: have the Cloudflare zone id for sovereign-node.link to hand (Overview page of the zone). A Zone:DNS:Edit-only token cannot look the zone up by name; Phase 1 step 7 asks for the id once if the token cannot list zones.</t>
+          <t>New in v0.3.2: /etc/atlas/secrets/smb.cred (root, mode 600; username=, password=, domain= lines) for the Windows share account; Phase 2 checks it at minute 0 and prints the command that creates it without the password touching a command line.</t>
         </is>
       </c>
       <c r="D11" s="16" t="n"/>
@@ -6645,14 +6743,10 @@
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Source reference recordings for Alaric's gravelly voice and, if the British male presets collide, Gideon's. Sourced. The Day 1 script names the directory they are copied into before Phase 2; if absent, both fall back to the nearest Kokoro preset and V7 is recorded as deferred, not failed.</t>
-        </is>
-      </c>
-      <c r="D12" s="16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>New in v0.3.2: decide D15 (Secure Boot and the TPM binding) before Phase 1 step 2.</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="n"/>
       <c r="E12" s="17" t="n"/>
     </row>
     <row r="13">
@@ -6666,7 +6760,7 @@
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Have a monitor and keyboard available for Phase 1 only, in case first boot needs a hand. Done.</t>
+          <t>Create the Google Cloud OAuth client for Gmail, Calendar and Drive, and be reachable for roughly five minutes during the Phase 2 pause (V20). Client created. The consent click itself still happens during Phase 2; Google requires the account owner to click Allow. The client must be of the Desktop app type (its JSON has a top-level installed key; a web key is the wrong type and Phase 2 stops at minute 0 saying so). Drop the JSON into /srv/atlas/staging/inbox/google-oauth-client.json once Phase 1 has created that folder.</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr">
@@ -6682,19 +6776,15 @@
       </c>
       <c r="B14" s="11" t="inlineStr">
         <is>
-          <t>Automated on the Principal's instruction, no action needed</t>
+          <t>Principal's actions — what is genuinely left</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Cloudflare token relocation and deletion of CLOUDFLARE.txt: Phase 2 step 6b (V23).</t>
-        </is>
-      </c>
-      <c r="D14" s="16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>New in v0.3.1: create a Hugging Face access token (read scope) and, with the same account, accept the licences of the gated models on huggingface.co: pyannote/speaker-diarization-3.1 and pyannote/segmentation-3.0 (V6), black-forest-labs/FLUX.1-dev and stabilityai/stable-audio-open-1.0 (Phase 4). Phase 2 asks for the token once at its start and stores it under /etc/atlas/secrets/; a 403 during a pull names the licence page to visit.</t>
+        </is>
+      </c>
+      <c r="D14" s="16" t="n"/>
       <c r="E14" s="17" t="n"/>
     </row>
     <row r="15">
@@ -6703,19 +6793,15 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Automated on the Principal's instruction, no action needed</t>
+          <t>Principal's actions — what is genuinely left</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Director aliases generated from names rather than confirmed one by one (D14).</t>
-        </is>
-      </c>
-      <c r="D15" s="16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>New in v0.3.1: have the Cloudflare zone id for sovereign-node.link to hand (Overview page of the zone). A Zone:DNS:Edit-only token cannot look the zone up by name; Phase 1 step 7 asks for the id once if the token cannot list zones.</t>
+        </is>
+      </c>
+      <c r="D15" s="16" t="n"/>
       <c r="E15" s="17" t="n"/>
     </row>
     <row r="16">
@@ -6724,12 +6810,12 @@
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>Build-side preconditions</t>
+          <t>Principal's actions — what is genuinely left</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Ubuntu Server 26.04.1 installed on the 4 TB drive; 8 TB drive unpartitioned. Done.</t>
+          <t>Source reference recordings for Alaric's gravelly voice and, if the British male presets collide, Gideon's. Sourced. Drop them as alaric.* and gideon.* (WAV, MP3 or M4A; step 5 converts to 16 kHz mono WAV) into /srv/atlas/staging/inbox/voice-references/ once Phase 1 has created the folder; if absent, both fall back to the nearest Kokoro preset and V7 is recorded as deferred, not failed.</t>
         </is>
       </c>
       <c r="D16" s="16" t="inlineStr">
@@ -6745,12 +6831,12 @@
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Build-side preconditions</t>
+          <t>Principal's actions — what is genuinely left</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>BIOS: UMA minimum, IOMMU on, fTPM on, Secure Boot disabled (D2). Done.</t>
+          <t>Have a monitor and keyboard available for Phase 1 only, in case first boot needs a hand. Done.</t>
         </is>
       </c>
       <c r="D17" s="16" t="inlineStr">
@@ -6766,12 +6852,12 @@
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Build-side preconditions</t>
+          <t>Automated on the Principal's instruction, no action needed</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>LAN address reserved for the node on the router, over Wi-Fi; UDP 51820 forward confirmed to that address. Done.</t>
+          <t>Cloudflare token relocation and deletion of CLOUDFLARE.txt: Phase 2 step 6b (V23).</t>
         </is>
       </c>
       <c r="D18" s="16" t="inlineStr">
@@ -6787,12 +6873,12 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Build-side preconditions</t>
+          <t>Automated on the Principal's instruction, no action needed</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>Internet bandwidth known, so the ~690 GB Phase 3 download can be planned. Done; the figure was not recorded in the workbook, so the 100 Mbps planning assumption in 15.4 stands until stated.</t>
+          <t>Director aliases generated from names rather than confirmed one by one (D14).</t>
         </is>
       </c>
       <c r="D19" s="16" t="inlineStr">
@@ -6808,12 +6894,12 @@
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Accepted resolutions</t>
+          <t>Build-side preconditions</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>C1 through C20 accepted in the returned workbook. C19 was reopened and re-decided in the Principal's favour.</t>
+          <t>Ubuntu Server 26.04.1 installed on the 4 TB drive with the installer's encrypted-LVM (LUKS) option (Section 3.5 requires both volumes encrypted; pre-flight stops on an unencrypted OS volume); 8 TB drive unpartitioned. Done per the returned workbook; confirm the encryption option was taken.</t>
         </is>
       </c>
       <c r="D20" s="16" t="inlineStr">
@@ -6829,12 +6915,12 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>Accepted resolutions</t>
+          <t>Build-side preconditions</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>C21 through C26, new in v0.2, accepted in the returned workbook: the Ubuntu and amd64v3 rejections, the quantisation rise, the closed reserve list, the vision consolidation, and the residency-versus-generation reading.</t>
+          <t>BIOS: UMA minimum, IOMMU on, fTPM on, Secure Boot disabled (D2). Done.</t>
         </is>
       </c>
       <c r="D21" s="16" t="inlineStr">
@@ -6850,24 +6936,108 @@
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
+          <t>Build-side preconditions</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>LAN address reserved for the node on the router, over Wi-Fi; UDP 51820 forward confirmed to that address. Done.</t>
+        </is>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Build-side preconditions</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>Internet bandwidth known, so the ~690 GB Phase 3 download can be planned. Done; the figure was not recorded in the workbook, so the 100 Mbps planning assumption in 15.4 stands until stated.</t>
+        </is>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
           <t>Accepted resolutions</t>
         </is>
       </c>
-      <c r="C22" s="11" t="inlineStr">
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>C1 through C20 accepted in the returned workbook. C19 was reopened and re-decided in the Principal's favour.</t>
+        </is>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Accepted resolutions</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>C21 through C26, new in v0.2, accepted in the returned workbook: the Ubuntu and amd64v3 rejections, the quantisation rise, the closed reserve list, the vision consolidation, and the residency-versus-generation reading.</t>
+        </is>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Accepted resolutions</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
         <is>
           <t>R9, R16, R19, R20 and R21 acknowledged in the returned workbook: two changed wording in v0.2, three were new.</t>
         </is>
       </c>
-      <c r="D22" s="16" t="inlineStr">
+      <c r="D26" s="16" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E22" s="17" t="n"/>
+      <c r="E26" s="17" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E22"/>
-  <conditionalFormatting sqref="D5:D22">
+  <autoFilter ref="A4:E26"/>
+  <conditionalFormatting sqref="D5:D26">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Yes"</formula>
     </cfRule>
@@ -6879,7 +7049,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="D5:D22" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Choose" prompt="Pick one: Yes / No / N/A" type="list" errorStyle="stop">
+    <dataValidation sqref="D5:D26" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Choose" prompt="Pick one: Yes / No / N/A" type="list" errorStyle="stop">
       <formula1>"Yes,No,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Baseline v0.3.4: R22 to R25 acknowledged by the Principal (workbook and Section 22)
The Principal acknowledged R22 to R25 on 2026-10-08: the docker-group
risk and the PCR 7 / Secure Boot risk (both v0.3.2), the xrdp exposure
and the unattended-reboot gap (both v0.3.4).

- Workbook sheet "3 Risks": every row now reads Yes; R22-R25 carry
  "Acknowledged 2026-10-08" in Notes. Summary and instructions no longer
  list them as outstanding; only the optional sheet 5 rows remain.
- Document: the Section 22 checklist row is ticked and the status line
  records the acknowledgement.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USyWZdFCwDpe3L4dpdaCcG
</commit_message>
<xml_diff>
--- a/docs/ATLAS_BUILD_BASELINE.xlsx
+++ b/docs/ATLAS_BUILD_BASELINE.xlsx
@@ -581,7 +581,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Companion to docs/ATLAS_FRAMEWORK_REVIEW.md v0.3.4 (2026-10-08). Ubuntu Server 26.04.1 re-confirmed over Fedora 44 KDE Plasma (C27). The Day 1 scripts are delivered under scripts/day1 and never stop on a missing input from the Principal (they ask once, defer, and keep a to-do list); this workbook carries the record of decisions and the four risk rows still to acknowledge. Nothing has been executed.</t>
+          <t>Companion to docs/ATLAS_FRAMEWORK_REVIEW.md v0.3.4 (2026-10-08). Ubuntu Server 26.04.1 re-confirmed over Fedora 44 KDE Plasma (C27). The Day 1 scripts are delivered under scripts/day1 and never stop on a missing input from the Principal (they ask once, defer, and keep a to-do list); every decision, resolution and risk is now confirmed; this workbook is the closed record, plus the optional pre-execution rows on sheet 5. Nothing has been executed.</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>1. Sheets 1, 2 and 3 are a record of your answers of 2026-09-21, 2026-10-05 (D15: Secure Boot enabled) and 2026-10-08 (C27: Ubuntu kept). Four rows still need you: R22 to R25 on sheet 3. Sheet 5 lists the one new precondition (Secure Boot on in the BIOS) and the optional items the scripts ask for at a prompt. Sheet 4 fills during Day 1.</t>
+          <t>1. Sheets 1, 2 and 3 are a record of your answers of 2026-09-21, 2026-10-05 (D15: Secure Boot enabled) and 2026-10-08 (C27: Ubuntu kept; R22 to R25 acknowledged). Nothing on them still needs you. Sheet 5 lists the one new precondition (Secure Boot on in the BIOS) and the optional items the scripts ask for at a prompt. Sheet 4 fills during Day 1.</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>6. Outstanding before Day 1: R22 to R25 and the blank sheet 5 rows (only the Secure Boot BIOS setting is required; the rest are optional and can be given at the prompt or left for the live ATLAS). To reopen any other item, change its response cell (Changed my mind, Disagree, Discuss or No) and write the reason beside it; the progress table below shows it at once.</t>
+          <t>6. Outstanding before Day 1: the blank sheet 5 rows (only the Secure Boot BIOS setting is required; the rest are optional and can be given at the prompt or left for the live ATLAS). To reopen any other item, change its response cell (Changed my mind, Disagree, Discuss or No) and write the reason beside it; the progress table below shows it at once.</t>
         </is>
       </c>
     </row>
@@ -5149,7 +5149,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Section 20. R1 to R21 acknowledged in the workbook returned 2026-09-21. R22 and R23 (v0.3.2) and R24 and R25 (v0.3.4: the xrdp exposure and the unattended-reboot gap) are blank; R23 is mitigated by D15 (Secure Boot enabled) once the BIOS setting is made.</t>
+          <t>Section 20. R1 to R21 acknowledged in the workbook returned 2026-09-21; R22 and R23 (v0.3.2) and R24 and R25 (v0.3.4: the xrdp exposure and the unattended-reboot gap) acknowledged by the Principal on 2026-10-08. R23 is mitigated by D15 (Secure Boot enabled) once the BIOS setting is made.</t>
         </is>
       </c>
     </row>
@@ -5612,8 +5612,16 @@
           <t>Accepted for Day 1 and recorded in every script header; Day 2 options are rootless Docker or a socket proxy that allows only the sandbox and engine images. New in v0.3.2</t>
         </is>
       </c>
-      <c r="F17" s="16" t="n"/>
-      <c r="G17" s="17" t="n"/>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G17" s="17" t="inlineStr">
+        <is>
+          <t>Acknowledged 2026-10-08</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
@@ -5641,8 +5649,16 @@
           <t>D15 closed as Secure Boot enabled (v0.3.3); mitigated once the Principal makes the BIOS setting. Until then pre-flight warns, V2 notes it and the to-do secure-boot is open; the enrolment itself proceeds. New in v0.3.2</t>
         </is>
       </c>
-      <c r="F18" s="16" t="n"/>
-      <c r="G18" s="17" t="n"/>
+      <c r="F18" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G18" s="17" t="inlineStr">
+        <is>
+          <t>Acknowledged 2026-10-08</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
@@ -5670,8 +5686,16 @@
           <t>v0.3.4: port 3389 only from the LAN subnet and WireGuard; the VNC proxy entry (vnc-any, the CVSS 9.8 CVE-2026-41252 path, also commented out upstream in 0.10.6.1), the NeutrinoRDP proxy entry (its module is not shipped) and Xvnc switched off; no root login, no alternate shell, TLS only; optional RDP_ALLOW_FROM (addresses inside the LAN, never the WireGuard bridge, checked before the firewall is touched) narrows the LAN side to the Principal's PC, and step 5b records the to-do with the LAN address the PC connected from. Residual: the remaining pre-login bugs from those hosts. Watch for a 26.04 xrdp security update; a later option is to keep 3389 on WireGuard only. New in v0.3.4</t>
         </is>
       </c>
-      <c r="F19" s="16" t="n"/>
-      <c r="G19" s="17" t="n"/>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G19" s="17" t="inlineStr">
+        <is>
+          <t>Acknowledged 2026-10-08</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
@@ -5699,8 +5723,16 @@
           <t>Accepted for Day 1: an automatic reboot would interrupt long jobs. Day 2: the live ATLAS reports "reboot required" and pending Docker CE/Chrome updates through ntfy and schedules the reboot with the Principal. New in v0.3.4</t>
         </is>
       </c>
-      <c r="F20" s="16" t="n"/>
-      <c r="G20" s="17" t="n"/>
+      <c r="F20" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G20" s="17" t="inlineStr">
+        <is>
+          <t>Acknowledged 2026-10-08</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
@@ -7177,10 +7209,14 @@
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>R22 to R25 to be acknowledged in the workbook (R22 and R23 new in v0.3.2, R24 and R25 new in v0.3.4).</t>
-        </is>
-      </c>
-      <c r="D29" s="16" t="n"/>
+          <t>R22 to R25 acknowledged by the Principal on 2026-10-08 (R22 and R23 new in v0.3.2, R24 and R25 new in v0.3.4).</t>
+        </is>
+      </c>
+      <c r="D29" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="E29" s="17" t="n"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
WIP checkpoint: open-input recommendations build in progress (S56)
Partial state while the build workflow runs: engine configuration for the
approved D-33/D-47 floors, D-16 profiles and the D-19/D-60 removals, with
download and network changes under way. Not yet reviewed or fully tested;
the completed, checked change follows in a later commit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USyWZdFCwDpe3L4dpdaCcG
</commit_message>
<xml_diff>
--- a/docs/ATLAS_BUILD_BASELINE.xlsx
+++ b/docs/ATLAS_BUILD_BASELINE.xlsx
@@ -581,7 +581,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Companion to docs/ATLAS_FRAMEWORK_REVIEW.md v0.4.0 (2026-10-17), built from it by scripts/day1/tools/build-baseline-workbook.py (D-27). v0.4.0 records the action register the Principal returned on 2026-10-16, every row approved as recommended (P-10 with the Principal's change: Eleanor's router stays at 4B for classification only, and her own persona work moves to GLM-5.3-Flash; the questions on P-10 and on memory headroom, N-01 and N-03, are answered in the document's 5.3, 4.1 and 4.2): llama.cpp re-pinned to build tag b11474, with the old pin v0.4.1 kept only for the output-parity test V25 (sheet 4); GLM-5.3-Flash UD-IQ4_XS (with its glm5v projector, also the vision engine and the long-document route) and DeepSeek-V4-Flash-0731 UD-Q8_K_XL (Arthur and the Apex) as the Day 1 seats, gpt-oss-120b as the fast utility and fallback floor, the 4B router unchanged; one LLM seat resident at a time; the Engine Arbiter budgeting exact file bytes; the Qwen3 4B embedder and reranker on the CPU, replacing the bge pair before Day 1; the Phase 3 pull cut to about 448 GB; and pyannote community-1 now (C-06). D16 to D27 on sheet 1 record the decisions (D16 to D18 reopen D4, D10 and D12) and C28 to C30 on sheet 2 supersede C23, C25 and C26; R29 to R33 on sheet 3, with R4, R17, R19 and R20 restated, were acknowledged by the Principal on 2026-10-17, the day the Principal also approved the six RAM fixes (S55: an explicit prompt-cache cap on every engine, a 4 GiB /tmp, at most 8 Celery cpu workers, memory caps on Kokoro, speaches and Docling, an order for the out-of-memory killer, and a seat whose start failed stopped before its reservation goes) and confirmed V25's pass marks, with no new version number. The specialist seats (Intern-S1, Ling-3.0-flash-Fin, Baichuan-M3, Qwen3-Coder-Next), slot save and restore, swap batching, the speech, image and OCR companions, the EmbeddingGemma 2 side index, the Qwen3.8-Flash-Next and Nemotron 3 Super pulls, the drafters and the DeepSeek V4.1 trial are phased after Day 1, each with its to-do; where an approved row leaves an input to the Principal (the decode floors, the context targets, the test sets), its default is built and a to-do raised (sheet 5). The uncensored-seat items (D-07, D-08, D-09, D-58, N-10, P-05, P-17, S-05) are unchanged by this revision and remain the Principal's to configure. Until v0.4.0 this workbook was the closed v0.3.5 record of 2026-10-12: Ubuntu Server kept over Fedora 44 KDE Plasma (C27), the crash-kernel memory reclaimed with panic=10 (S48), kexec handover off (S49), the hardware watchdog (S50), torchaudio pinned so Phase 4 stays on ROCm 10.0.0 (S51), every request kept inside its engine's slot with the Phase 3 memory records (S52), and the pruning fixes (S53), with every decision and resolution confirmed and every risk acknowledged. The Day 1 scripts under scripts/day1 never stop on a missing input from the Principal (they ask once, defer, and keep a to-do list). Nothing has been executed.</t>
+          <t>Companion to docs/ATLAS_FRAMEWORK_REVIEW.md v0.4.0 (2026-10-17), built from it by scripts/day1/tools/build-baseline-workbook.py (D-27). v0.4.0 records the action register the Principal returned on 2026-10-16, every row approved as recommended (P-10 with the Principal's change: Eleanor's router stays at 4B for classification only, and her own persona work moves to GLM-5.3-Flash; the questions on P-10 and on memory headroom, N-01 and N-03, are answered in the document's 5.3, 4.1 and 4.2): llama.cpp re-pinned to build tag b11474, with the old pin v0.4.1 kept only for the output-parity test V25 (sheet 4); GLM-5.3-Flash UD-IQ4_XS (with its glm5v projector, also the vision engine and the long-document route) and DeepSeek-V4-Flash-0731 UD-Q8_K_XL (Arthur and the Apex) as the Day 1 seats, gpt-oss-120b as the fast utility and fallback floor, the 4B router unchanged; one LLM seat resident at a time; the Engine Arbiter budgeting exact file bytes; the Qwen3 4B embedder and reranker on the CPU, replacing the bge pair before Day 1; the Phase 3 pull cut to about 448 GB; and pyannote community-1 now (C-06). D16 to D27 on sheet 1 record the decisions (D16 to D18 reopen D4, D10 and D12) and C28 to C30 on sheet 2 supersede C23, C25 and C26; R29 to R33 on sheet 3, with R4, R17, R19 and R20 restated, were acknowledged by the Principal on 2026-10-17, the day the Principal also approved the six RAM fixes (S55: an explicit prompt-cache cap on every engine, a 4 GiB /tmp, at most 8 Celery cpu workers, memory caps on Kokoro, speaches and Docling, an order for the out-of-memory killer, and a seat whose start failed stopped before its reservation goes) and confirmed V25's pass marks, with no new version number. The specialist seats (Intern-S1, Ling-3.0-flash-Fin, Baichuan-M3), slot save and restore, swap batching, the speech, image and OCR companions, the Qwen3.8-Flash-Next and Nemotron 3 Super pulls, the drafters and the DeepSeek V4.1 trial are phased after Day 1, each with its to-do; where an approved row leaves an input to the Principal (the decode floors, the context targets, the test sets), its default is built and a to-do raised (sheet 5). The uncensored-seat items (D-07, D-08, D-09, D-58, N-10, P-05, P-17, S-05) are unchanged by this revision and remain the Principal's to configure. Until v0.4.0 this workbook was the closed v0.3.5 record of 2026-10-12: Ubuntu Server kept over Fedora 44 KDE Plasma (C27), the crash-kernel memory reclaimed with panic=10 (S48), kexec handover off (S49), the hardware watchdog (S50), torchaudio pinned so Phase 4 stays on ROCm 10.0.0 (S51), every request kept inside its engine's slot with the Phase 3 memory records (S52), and the pruning fixes (S53), with every decision and resolution confirmed and every risk acknowledged. The Day 1 scripts under scripts/day1 never stop on a missing input from the Principal (they ask once, defer, and keep a to-do list). Nothing has been executed.</t>
         </is>
       </c>
     </row>
@@ -12562,7 +12562,7 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>v0.4.0 (S-29, D-37): owners and tiers unchanged. A preset reaches a seat only through its owner's binding or its engine field, never a domain card; on Day 1 only TF_OMEGA carries one (deepseek-v4-flash, the Apex), and every other preset runs on its owner's default engine (GLM-5.3-Flash for every director but Valerie, whose engine is unchanged). The phased engines a preset will carry are named in task-forces.json notes: Ling-3.0-flash-Fin on TF_GAMMA, TF_DELTA and TF_EPSILON, Qwen3-Coder-Next on TF_MU, Baichuan-M3 and Intern-S1 on TF_UPSILON. No new prefix.</t>
+          <t>v0.4.0 (S-29, D-37): owners and tiers unchanged. A preset reaches a seat only through its owner's binding or its engine field, never a domain card; on Day 1 only TF_OMEGA carries one (deepseek-v4-flash, the Apex), and every other preset runs on its owner's default engine (GLM-5.3-Flash for every director but Valerie, whose engine is unchanged). The phased engines a preset will carry are named in task-forces.json notes: Ling-3.0-flash-Fin on TF_GAMMA, TF_DELTA and TF_EPSILON, Baichuan-M3 and Intern-S1 on TF_UPSILON; TF_MU has none, since D-19 (c) dropped Qwen3-Coder-Next on 2026-10-17. No new prefix.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
WIP checkpoint: jurisdictions and live-ATLAS inputs in progress (S57)
Partial state while the follow-up workflow runs: Commonwealth, VIC, NSW and QLD
coverage in the domain profiles and cards, the standards-licensing rule, the
live MedGemma acceptance flow and live briefs. The legal citations are still
under review; the checked change follows in a later commit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01USyWZdFCwDpe3L4dpdaCcG
</commit_message>
<xml_diff>
--- a/docs/ATLAS_BUILD_BASELINE.xlsx
+++ b/docs/ATLAS_BUILD_BASELINE.xlsx
@@ -28,7 +28,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2 Resolutions'!$A$4:$E$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3 Risks'!$A$4:$G$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4 Verification'!$A$4:$E$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5 Checklist'!$A$4:$E$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5 Checklist'!$A$4:$E$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -581,7 +581,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Companion to docs/ATLAS_FRAMEWORK_REVIEW.md v0.4.0 (2026-10-17), built from it by scripts/day1/tools/build-baseline-workbook.py (D-27). v0.4.0 records the action register the Principal returned on 2026-10-16, every row approved as recommended (P-10 with the Principal's change: Eleanor's router stays at 4B for classification only, and her own persona work moves to GLM-5.3-Flash; the questions on P-10 and on memory headroom, N-01 and N-03, are answered in the document's 5.3, 4.1 and 4.2): llama.cpp re-pinned to build tag b11474, with the old pin v0.4.1 kept only for the output-parity test V25 (sheet 4); GLM-5.3-Flash UD-IQ4_XS (with its glm5v projector, also the vision engine and the long-document route) and DeepSeek-V4-Flash-0731 UD-Q8_K_XL (Arthur and the Apex) as the Day 1 seats, gpt-oss-120b as the fast utility and fallback floor, the 4B router unchanged; one LLM seat resident at a time; the Engine Arbiter budgeting exact file bytes; the Qwen3 4B embedder and reranker on the CPU, replacing the bge pair before Day 1; the Phase 3 pull cut to about 448 GB; and pyannote community-1 now (C-06). D16 to D27 on sheet 1 record the decisions (D16 to D18 reopen D4, D10 and D12) and C28 to C30 on sheet 2 supersede C23, C25 and C26; R29 to R33 on sheet 3, with R4, R17, R19 and R20 restated, were acknowledged by the Principal on 2026-10-17, the day the Principal also approved the six RAM fixes (S55: an explicit prompt-cache cap on every engine, a 4 GiB /tmp, at most 8 Celery cpu workers, memory caps on Kokoro, speaches and Docling, an order for the out-of-memory killer, and a seat whose start failed stopped before its reservation goes) and confirmed V25's pass marks, with no new version number. The specialist seats (Intern-S1, Ling-3.0-flash-Fin, Baichuan-M3), slot save and restore, swap batching, the speech, image and OCR companions, the Qwen3.8-Flash-Next and Nemotron 3 Super pulls, the drafters and the DeepSeek V4.1 trial are phased after Day 1, each with its to-do; where an approved row leaves an input to the Principal (the decode floors, the context targets, the test sets), its default is built and a to-do raised (sheet 5). Later on 2026-10-17 (S56) the Principal approved the recommendations for those inputs: decode floors at 8k (gpt-oss-120b 25, GLM-5.3-Flash 6, DeepSeek-V4-Flash-0731 4, the router 20 tok/s) with prefill floors and placement checks, the D-16 profile of the phased medical and science seats, no dedicated coder seat (Qwen3-Coder-Next not pulled), EmbeddingGemma 2 dropped, MedGemma 1.5 4B only on conditions, and the designs of the seat test sets and the V4.1 trial set; and recorded a 2,000 Mbps line with the node moving to a cable on its 10 GbE port before Phase 1. What those answers still leave open is on sheet 5. The uncensored-seat items (D-07, D-08, D-09, D-58, N-10, P-05, P-17, S-05) are unchanged by this revision and remain the Principal's to configure. Until v0.4.0 this workbook was the closed v0.3.5 record of 2026-10-12: Ubuntu Server kept over Fedora 44 KDE Plasma (C27), the crash-kernel memory reclaimed with panic=10 (S48), kexec handover off (S49), the hardware watchdog (S50), torchaudio pinned so Phase 4 stays on ROCm 10.0.0 (S51), every request kept inside its engine's slot with the Phase 3 memory records (S52), and the pruning fixes (S53), with every decision and resolution confirmed and every risk acknowledged. The Day 1 scripts under scripts/day1 never stop on a missing input from the Principal (they ask once, defer, and keep a to-do list). Nothing has been executed.</t>
+          <t>Companion to docs/ATLAS_FRAMEWORK_REVIEW.md v0.4.0 (2026-10-17), built from it by scripts/day1/tools/build-baseline-workbook.py (D-27). v0.4.0 records the action register the Principal returned on 2026-10-16, every row approved as recommended (P-10 with the Principal's change: Eleanor's router stays at 4B for classification only, and her own persona work moves to GLM-5.3-Flash; the questions on P-10 and on memory headroom, N-01 and N-03, are answered in the document's 5.3, 4.1 and 4.2): llama.cpp re-pinned to build tag b11474, with the old pin v0.4.1 kept only for the output-parity test V25 (sheet 4); GLM-5.3-Flash UD-IQ4_XS (with its glm5v projector, also the vision engine and the long-document route) and DeepSeek-V4-Flash-0731 UD-Q8_K_XL (Arthur and the Apex) as the Day 1 seats, gpt-oss-120b as the fast utility and fallback floor, the 4B router unchanged; one LLM seat resident at a time; the Engine Arbiter budgeting exact file bytes; the Qwen3 4B embedder and reranker on the CPU, replacing the bge pair before Day 1; the Phase 3 pull cut to about 448 GB; and pyannote community-1 now (C-06). D16 to D27 on sheet 1 record the decisions (D16 to D18 reopen D4, D10 and D12) and C28 to C30 on sheet 2 supersede C23, C25 and C26; R29 to R33 on sheet 3, with R4, R17, R19 and R20 restated, were acknowledged by the Principal on 2026-10-17, the day the Principal also approved the six RAM fixes (S55: an explicit prompt-cache cap on every engine, a 4 GiB /tmp, at most 8 Celery cpu workers, memory caps on Kokoro, speaches and Docling, an order for the out-of-memory killer, and a seat whose start failed stopped before its reservation goes) and confirmed V25's pass marks, with no new version number. The specialist seats (Intern-S1, Ling-3.0-flash-Fin, Baichuan-M3), slot save and restore, swap batching, the speech, image and OCR companions, the Qwen3.8-Flash-Next and Nemotron 3 Super pulls, the drafters and the DeepSeek V4.1 trial are phased after Day 1, each with its to-do; where an approved row leaves an input to the Principal (the decode floors, the context targets, the test sets), its default is built and a to-do raised (sheet 5). Later on 2026-10-17 (S56) the Principal approved the recommendations for those inputs: decode floors at 8k (gpt-oss-120b 25, GLM-5.3-Flash 6, DeepSeek-V4-Flash-0731 4, the router 20 tok/s) with prefill floors and placement checks, the D-16 profile of the phased medical and science seats, no dedicated coder seat (Qwen3-Coder-Next not pulled), EmbeddingGemma 2 dropped, MedGemma 1.5 4B only on conditions, and the designs of the seat test sets and the V4.1 trial set; and recorded a 2,000 Mbps line with the node moving to a cable on its 10 GbE port before Phase 1. What those answers still leave open is on sheet 5. The same day (S57) the Principal's statements were recorded: ATLAS's Australian law is that of the Commonwealth, VIC, NSW and QLD; an Australian Standard's text is held only under the Principal's own licence, otherwise its number, edition and free commentary; the briefs for the seat test sets are collected once ATLAS is live, from real examples; and the MedGemma licence decision is a task for the live ATLAS with the Principal present. Two proposals await the Principal, not decided: the 16 Australian-law tasks spread across the four jurisdictions, and about 10 Australian tax and finance tasks. The uncensored-seat items (D-07, D-08, D-09, D-58, N-10, P-05, P-17, S-05) are unchanged by this revision and remain the Principal's to configure. Until v0.4.0 this workbook was the closed v0.3.5 record of 2026-10-12: Ubuntu Server kept over Fedora 44 KDE Plasma (C27), the crash-kernel memory reclaimed with panic=10 (S48), kexec handover off (S49), the hardware watchdog (S50), torchaudio pinned so Phase 4 stays on ROCm 10.0.0 (S51), every request kept inside its engine's slot with the Phase 3 memory records (S52), and the pruning fixes (S53), with every decision and resolution confirmed and every risk acknowledged. The Day 1 scripts under scripts/day1 never stop on a missing input from the Principal (they ask once, defer, and keep a to-do list). Nothing has been executed.</t>
         </is>
       </c>
     </row>
@@ -595,7 +595,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>1. Sheets 1, 2 and 3 are a record of your answers of 2026-09-21, 2026-10-05 (D15: Secure Boot enabled), 2026-10-08 (C27: Ubuntu kept; R22 to R25 acknowledged), 2026-10-13 (R26 to R28 acknowledged), 2026-10-16 (the action register: D16 to D27 and C28 to C30) and 2026-10-17 (R29 to R33 and the restated R4, R17, R19 and R20 acknowledged; later, S56: your answers to the open inputs in D16 to D26, R9 and R20 restated with B-27). Nothing on them needs you now. Sheet 5 records the Secure Boot BIOS setting made and the USB recovery drive in hand (both confirmed 2026-10-13) and lists the optional items the scripts ask for at a prompt and the inputs still left to you, each with the default already built. Sheet 4 fills during Day 1.</t>
+          <t>1. Sheets 1, 2 and 3 are a record of your answers of 2026-09-21, 2026-10-05 (D15: Secure Boot enabled), 2026-10-08 (C27: Ubuntu kept; R22 to R25 acknowledged), 2026-10-13 (R26 to R28 acknowledged), 2026-10-16 (the action register: D16 to D27 and C28 to C30) and 2026-10-17 (R29 to R33 and the restated R4, R17, R19 and R20 acknowledged; later, S56: your answers to the open inputs in D16 to D26, R9 and R20 restated with B-27; S57: in D20, the briefs collected once ATLAS is live). Nothing on them needs you now. Sheet 5 records the Secure Boot BIOS setting made and the USB recovery drive in hand (both confirmed 2026-10-13) and lists the optional items the scripts ask for at a prompt and the inputs still left to you, each with the default already built. Sheet 4 fills during Day 1.</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>6. Outstanding before Phase 1: sheet 5 row 31, the cable (your choice of 2026-10-17, S56): plug it into the 10 GbE port not marked DASH and a 2.5 GbE router port, move the reservation and the UDP 51820 forward to that port's MAC and take Wi-Fi off the LAN subnet (pre-flight warns, never stops, if it is not done). The other blank sheet 5 rows are optional or wait until after Day 1, and can be given at the prompt or left for the live ATLAS; sheet 5 row 28 still asks you to confirm that the installer's encryption option was taken (if it was not, Day 1 warns and records a to-do, never a stop). To reopen any other item, change its response cell (Changed my mind, Disagree, Discuss or No) and write the reason beside it; the progress table below shows it at once.</t>
+          <t>6. Outstanding before Phase 1: sheet 5 row 32, the cable (your choice of 2026-10-17, S56): plug it into the 10 GbE port not marked DASH and a 2.5 GbE router port, move the reservation and the UDP 51820 forward to that port's MAC and take Wi-Fi off the LAN subnet (pre-flight warns, never stops, if it is not done). The other blank sheet 5 rows are optional or wait until after Day 1, and can be given at the prompt or left for the live ATLAS; sheet 5 row 29 still asks you to confirm that the installer's encryption option was taken (if it was not, Day 1 warns and records a to-do, never a stop). To reopen any other item, change its response cell (Changed my mind, Disagree, Discuss or No) and write the reason beside it; the progress table below shows it at once.</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>COUNTA('5 Checklist'!$A$5:$A$45)</f>
+        <f>COUNTA('5 Checklist'!$A$5:$A$46)</f>
         <v/>
       </c>
       <c r="C25" s="12">
@@ -872,7 +872,7 @@
         <v/>
       </c>
       <c r="D25" s="12">
-        <f>COUNTIF('5 Checklist'!$D$5:$D$45,"Yes")+COUNTIF('5 Checklist'!$D$5:$D$45,"N/A")</f>
+        <f>COUNTIF('5 Checklist'!$D$5:$D$46,"Yes")+COUNTIF('5 Checklist'!$D$5:$D$46,"N/A")</f>
         <v/>
       </c>
       <c r="E25" s="12">
@@ -880,11 +880,11 @@
         <v/>
       </c>
       <c r="F25" s="12">
-        <f>COUNTIF('5 Checklist'!$D$5:$D$45,"No")</f>
+        <f>COUNTIF('5 Checklist'!$D$5:$D$46,"No")</f>
         <v/>
       </c>
       <c r="G25" s="12">
-        <f>COUNTBLANK('5 Checklist'!$D$5:$D$45)</f>
+        <f>COUNTBLANK('5 Checklist'!$D$5:$D$46)</f>
         <v/>
       </c>
     </row>
@@ -2266,7 +2266,7 @@
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Green. *S56 (C-12, approved by the Principal on 2026-10-17):* Rad-DINO alone. MedGemma 1.5 4B joins it as an on-demand imaging tool, a companion and not an LLM seat, never resident, only once three things hold: the Principal accepts Google's HAI-DEF terms (an open box, Section 22); a new non-seat Arbiter class is built and tested, so that a read evicts the resident seat only for memory, never by seat exclusivity; and a node test shows its reads beat GLM-5.3-Flash's own vision on the same public cases. Then: BF16 weights (7.77 GB) with the BF16 mmproj (0.85 GB) from unsloth/medgemma-1.5-4b-it-GGUF, Q8_0 (4.13 GB) as the fallback, 1 × 32,768, about 10.8 GiB projected (INFERRED); each read a preliminary draft that Minerva's seat reasons over, never sent to the Principal unreviewed; reads batched so GLM is evicted at most once per batch. The terms, in brief (VERIFIED, fetched 2026-10-17): they bind every copy, the ungated unsloth GGUF included; no diagnosis and no automated healthcare decision (a licensed clinician decides); no serving to anyone else; other people's images, family members' included, only with their consent; the Principal indemnifies Google; Google may terminate, and every copy is then deleted; California law. Rad-DINO stays research-use only per its card</t>
+          <t>Green. *S56 (C-12, approved by the Principal on 2026-10-17):* Rad-DINO alone. MedGemma 1.5 4B joins it as an on-demand imaging tool, a companion and not an LLM seat, never resident, only once three things hold: the Principal accepts Google's HAI-DEF terms (an open box, Section 22); a new non-seat Arbiter class is built and tested, so that a read evicts the resident seat only for memory, never by seat exclusivity; and a node test shows its reads beat GLM-5.3-Flash's own vision on the same public cases. Then: BF16 weights (7.77 GB) with the BF16 mmproj (0.85 GB) from unsloth/medgemma-1.5-4b-it-GGUF, Q8_0 (4.13 GB) as the fallback, 1 × 32,768, about 10.8 GiB projected (INFERRED); each read a preliminary draft that Minerva's seat reasons over, never sent to the Principal unreviewed; reads batched so GLM is evicted at most once per batch. The terms, in brief (VERIFIED, fetched 2026-10-17): they bind every copy, the ungated unsloth GGUF included; no diagnosis and no automated healthcare decision (a licensed clinician decides); no serving to anyone else; other people's images, family members' included, only with their consent; the Principal indemnifies Google; Google may terminate, and every copy is then deleted; California law. *S57 (the Principal, 2026-10-17):* the licence decision is a task for the live ATLAS, with the Principal present to approve. After Day 1 ATLAS raises it and shows a plain summary of the HAI-DEF Terms of Use and Prohibited Use Policy, with their links (https://developers.google.com/health-ai-developer-foundations/terms and https://developers.google.com/health-ai-developer-foundations/prohibited-use-policy). The Principal decides. On a yes, the Principal accepts on the model's Hugging Face page (google/medgemma-1.5-4b-it, gated; VERIFIED 2026-10-17) with their own account; ATLAS never accepts for them (16.3 item 2). ATLAS then records the date and the terms version in the ledger (on 2026-10-17 the two pages read "Last modified" 15 and 14 November 2024, VERIFIED), pulls MedGemma 1.5 4B and runs the node test against GLM-5.3-Flash's own vision; the Arbiter-class condition above still applies. On a no, Rad-DINO alone. Rad-DINO stays research-use only per its card</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
@@ -2499,7 +2499,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>v0.4.0: Qwen2.5-VL-72B and Meditron-70B are retired, their rows kept as the record: the vision engine is GLM-5.3-Flash with its glm5v projector, a Phase 3 GGUF engine, and Minerva's cross-check moves to the phased Baichuan-M3. The image tier (Z-Image-Turbo, Qwen-Image-2512) is phased after Day 1 (T-25). Rad-DINO stands alone until MedGemma 1.5 4B's conditions hold: the Principal's acceptance of the HAI-DEF terms, a non-seat Arbiter class and a node test against GLM-5.3-Flash's own vision (C-12, S56).</t>
+          <t>v0.4.0: Qwen2.5-VL-72B and Meditron-70B are retired, their rows kept as the record: the vision engine is GLM-5.3-Flash with its glm5v projector, a Phase 3 GGUF engine, and Minerva's cross-check moves to the phased Baichuan-M3. The image tier (Z-Image-Turbo, Qwen-Image-2512) is phased after Day 1 (T-25). Rad-DINO stands alone until MedGemma 1.5 4B's conditions hold: the Principal's acceptance of the HAI-DEF terms, a non-seat Arbiter class and a node test against GLM-5.3-Flash's own vision (C-12, S56). Since S57 the decision is a task for the live ATLAS with the Principal present: on a yes the Principal accepts on the model's Hugging Face page with their own account, and ATLAS never accepts for them.</t>
         </is>
       </c>
     </row>
@@ -3223,7 +3223,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Section 16. The never-without-the-Principal list is decision D8; the approval tiers are agreed. v0.4.0 adds standing rules 9 (routed engines use only lossless accelerations, S-50) and 10 (the arsenal admission rules, S-13).</t>
+          <t>Section 16. The never-without-the-Principal list is decision D8; the approval tiers are agreed. v0.4.0 adds standing rules 9 (routed engines use only lossless accelerations, S-50) and 10 (the arsenal admission rules, S-13). S57: item 2 covers every licence and terms of use; ATLAS never accepts terms on the Principal's behalf.</t>
         </is>
       </c>
     </row>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="D76" s="11" t="inlineStr">
         <is>
-          <t>*S56 (D-49):* the 100-task set in two waves of 50, drafted on the node by ATLAS and approved by the Principal, answered and judged blind through the evaluation runner (atlas-admin eval, built, phased; 6.2). A to-do for the Principal: the briefs, states and standards (Section 22); until the sets are scored GLM-5.3-Flash carries those seats unproven</t>
+          <t>*S56 (D-49):* the 100-task set in two waves of 50, drafted on the node by ATLAS and approved by the Principal, answered and judged blind through the evaluation runner (atlas-admin eval, built, phased; 6.2). A to-do for the Principal: the briefs and the standards list (Section 22). *S57:* the briefs are collected once ATLAS is live, from real examples as the work progresses, and the states are answered (VIC, NSW and QLD, with the Commonwealth); until the sets are scored GLM-5.3-Flash carries those seats unproven</t>
         </is>
       </c>
     </row>
@@ -5567,7 +5567,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Section 19. All twenty-seven are closed. D15 (Secure Boot and the TPM binding) was decided on 2026-10-05 as option (a), Secure Boot enabled in the BIOS. D16 to D27 (v0.4.0) record the action register the Principal returned on 2026-10-16, every row approved as recommended (P-10 with the Principal's change); D16, D17 and D18 reopen D4 (the retrieval models), D10 (the vision engine) and D12 (Meditron), whose rows say so in their Note. D16, D18, D20, D22, D24 and D26 carry the Principal's answers of 2026-10-17 to the inputs they had left open (S56: the decode, prefill and deep-tier floors, the D-16 profile, no dedicated coder seat, EmbeddingGemma 2 dropped, the test-set and trial designs).</t>
+          <t>Section 19. All twenty-seven are closed. D15 (Secure Boot and the TPM binding) was decided on 2026-10-05 as option (a), Secure Boot enabled in the BIOS. D16 to D27 (v0.4.0) record the action register the Principal returned on 2026-10-16, every row approved as recommended (P-10 with the Principal's change); D16, D17 and D18 reopen D4 (the retrieval models), D10 (the vision engine) and D12 (Meditron), whose rows say so in their Note. D16, D18, D20, D22, D24 and D26 carry the Principal's answers of 2026-10-17 to the inputs they had left open (S56: the decode, prefill and deep-tier floors, the D-16 profile, no dedicated coder seat, EmbeddingGemma 2 dropped, the test-set and trial designs). D20 also records S57: the D-49 briefs are collected once ATLAS is live, from real examples.</t>
         </is>
       </c>
     </row>
@@ -6148,7 +6148,7 @@
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>GLM-5.3-Flash UD-IQ4_XS for the professional seats, vision and long documents, provisional until the KLD run (D-02 option (c), D-10 option (a)); DeepSeek-V4-Flash-0731 UD-Q8_K_XL for Arthur and the Apex (D-11 option (a), D-13 option (b)); gpt-oss-120b as the fast utility and fallback floor, on its F16-trunk file (D-12 option (a), D-59 option (b)); Qwen3.5-122B-A10B retired (D-21 option (a)); the Deep Think pair GLM-5.3-Flash and DeepSeek-V4-Flash-0731 (D-22 option (a)); the cache at f16 where it is cheap, q8_0 elsewhere, q4_0 nowhere, GLM's provisional until T-04 (D-29 option (a)); a fixed reasoning setting per seat, chosen after the Phase 3 quality and KLD runs (T-03, to-do kld-run), with the vendor sampling recorded in each engines.json entry (D-30 option (b)); provisional Day 1 settings: DeepSeek-V4-Flash-0731 reasoning on at high effort, gpt-oss-120b high effort; dense 70B to 123B and 3-bit-only engines excluded (D-24 option (a)) and Mistral Large 2 Uncensored rejected (D-06 option (a)); test sets for the seats with no benchmark (D-49 option (a); the set design approved on 2026-10-17, S56, and the Principal's briefs a to-do)</t>
+          <t>GLM-5.3-Flash UD-IQ4_XS for the professional seats, vision and long documents, provisional until the KLD run (D-02 option (c), D-10 option (a)); DeepSeek-V4-Flash-0731 UD-Q8_K_XL for Arthur and the Apex (D-11 option (a), D-13 option (b)); gpt-oss-120b as the fast utility and fallback floor, on its F16-trunk file (D-12 option (a), D-59 option (b)); Qwen3.5-122B-A10B retired (D-21 option (a)); the Deep Think pair GLM-5.3-Flash and DeepSeek-V4-Flash-0731 (D-22 option (a)); the cache at f16 where it is cheap, q8_0 elsewhere, q4_0 nowhere, GLM's provisional until T-04 (D-29 option (a)); a fixed reasoning setting per seat, chosen after the Phase 3 quality and KLD runs (T-03, to-do kld-run), with the vendor sampling recorded in each engines.json entry (D-30 option (b)); provisional Day 1 settings: DeepSeek-V4-Flash-0731 reasoning on at high effort, gpt-oss-120b high effort; dense 70B to 123B and 3-bit-only engines excluded (D-24 option (a)) and Mistral Large 2 Uncensored rejected (D-06 option (a)); test sets for the seats with no benchmark (D-49 option (a); the set design approved on 2026-10-17, S56, and the Principal's briefs a to-do, collected once ATLAS is live from real examples, S57)</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
@@ -9092,7 +9092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -9112,7 +9112,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Section 22. The original rows were ticked in the workbook returned 2026-09-21; the rows added or reopened since were closed as each records: D15 decided and the Windows share deferred on 2026-10-05, C27 decided and R22 to R25 acknowledged by the Principal on 2026-10-08, the Secure Boot BIOS setting, the USB recovery drive and R26 to R28 ticked in the workbook returned 2026-10-13, and the action register, its licences, C28 to C30 and D16 to D27 ticked on 2026-10-16 (v0.4.0), R29 to R33 with the restated R4, R17, R19 and R20 acknowledged on 2026-10-17, and later that day the answers to the open inputs, the bandwidth and R9 and R20 as restated (S56). Blank rows: the optional items the scripts ask for at a prompt (Yes when provided, N/A to leave them for the live ATLAS to-do list); the inputs still left to the Principal, each already built with its stated default and kept as a to-do (the seat profiles and reasoning settings, the HAI-DEF decision for MedGemma, and after Day 1 the briefs for the seat test sets, the TF_OMEGA situations and the T-03 coding tasks); and the optional 60-second download test. One row is to do before Phase 1: row 31, the cable on the 10 GbE port not marked DASH, with the reservation and the forward moved to its MAC and Wi-Fi off the LAN subnet (S56; pre-flight warns, never stops, if it is not done). The Secure Boot row and the install rows are ticked. One request still stands on row 28, to confirm that the installer's encryption option (Encrypt the LVM group with LUKS) was taken; pre-flight checks the OS volume on Day 1, and an unencrypted one is a warning and the to-do os-volume-encryption, never a stop.</t>
+          <t>Section 22. The original rows were ticked in the workbook returned 2026-09-21; the rows added or reopened since were closed as each records: D15 decided and the Windows share deferred on 2026-10-05, C27 decided and R22 to R25 acknowledged by the Principal on 2026-10-08, the Secure Boot BIOS setting, the USB recovery drive and R26 to R28 ticked in the workbook returned 2026-10-13, and the action register, its licences, C28 to C30 and D16 to D27 ticked on 2026-10-16 (v0.4.0), R29 to R33 with the restated R4, R17, R19 and R20 acknowledged on 2026-10-17, and later that day the answers to the open inputs, the bandwidth and R9 and R20 as restated (S56). S57 records the Principal's statements the same day: the states answered (VIC, NSW and QLD, with the Commonwealth), the briefs collected once ATLAS is live, the standards list a new open row, and the MedGemma decision a task for the live ATLAS with the Principal present. Blank rows: the optional items the scripts ask for at a prompt (Yes when provided, N/A to leave them for the live ATLAS to-do list); the inputs still left to the Principal, each already built with its stated default and kept as a to-do (the seat profiles and reasoning settings; the HAI-DEF decision for MedGemma, taken with the live ATLAS; and after Day 1 the briefs for the seat test sets, from real examples, the standards list, the TF_OMEGA situations and the T-03 coding tasks); and the optional 60-second download test. One row is to do before Phase 1: row 32, the cable on the 10 GbE port not marked DASH, with the reservation and the forward moved to its MAC and Wi-Fi off the LAN subnet (S56; pre-flight warns, never stops, if it is not done). The Secure Boot row and the install rows are ticked. One request still stands on row 29, to confirm that the installer's encryption option (Encrypt the LVM group with LUKS) was taken; pre-flight checks the OS volume on Day 1, and an unencrypted one is a warning and the to-do os-volume-encryption, never a stop.</t>
         </is>
       </c>
     </row>
@@ -9495,7 +9495,7 @@
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Open, the Principal's decision (S56, C-12): accept or decline Google's HAI-DEF Terms of Use and Prohibited Use Policy for MedGemma 1.5 4B, recorded in the ledger like pyannote's. Accepting means no diagnosis, a licensed clinician making any real decision, no serving to anyone else, family members' images only with their consent, an indemnity to Google, and every copy deleted if Google terminates (California law). Declining, or leaving it, keeps Rad-DINO alone, with GLM-5.3-Flash's own vision reading scans (15.2).</t>
+          <t>Open, a task for the live ATLAS with the Principal present (S56, C-12; S57): accept or decline Google's HAI-DEF Terms of Use and Prohibited Use Policy for MedGemma 1.5 4B. Not needed for Day 1. After Day 1 ATLAS raises it and shows a plain summary of both, with their links (15.2); no script raises it on Day 1. The Principal decides. On a yes, the Principal accepts on the model's Hugging Face page with their own account, never ATLAS (16.3 item 2); ATLAS records the date and the terms version in the ledger, like pyannote's, then pulls MedGemma 1.5 4B and runs the node test against GLM-5.3-Flash's own vision. Accepting means no diagnosis, a licensed clinician making any real decision, no serving to anyone else, family members' images only with their consent, an indemnity to Google, and every copy deleted if Google terminates (California law). Declining, or leaving it, keeps Rad-DINO alone, with GLM-5.3-Flash's own vision reading scans (15.2).</t>
         </is>
       </c>
       <c r="D22" s="16" t="n"/>
@@ -9529,7 +9529,7 @@
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Open, after Day 1 (v0.4.0; the set design approved on 2026-10-17, S56): for the test sets of Australian law, HR, aviation, logistics, AEC, SCADA, game design, growth marketing, customer success and physical security / OSINT: a brief of about 15 minutes per domain (the 3 to 5 kinds of task you would give that seat, and 2 or 3 redacted real examples where they exist, which stay on the node); your state or states of operation (NSW and VIC are assumed); which paywalled standards you hold; then approval or edits of ATLAS's drafts, wave by wave, and blind grades for the escalations and the 10% calibration sample (D-49 option (a), T-27; to-do seat-test-sets). Until the sets are scored, GLM-5.3-Flash carries those seats unproven (6.2).</t>
+          <t>Open, after Day 1 (v0.4.0; the set design approved on 2026-10-17, S56; S57): for the test sets of Australian law, HR, aviation, logistics, AEC, SCADA, game design, growth marketing, customer success and physical security / OSINT: a brief of about 15 minutes per domain (the 3 to 5 kinds of task you would give that seat, and 2 or 3 redacted real examples where they exist, which stay on the node), collected once ATLAS is live, from real examples as the work progresses (the Principal, 2026-10-17); the standards list (the box below); then approval or edits of ATLAS's drafts, wave by wave, and blind grades for the escalations and the 10% calibration sample (D-49 option (a), T-27; to-do seat-test-sets). Your states of operation are answered: VIC, NSW and QLD, with the Commonwealth (S57, Section 1). Awaiting the Principal, not decided: spreading wave 1's 16 Australian-law tasks across the Commonwealth, VIC, NSW and QLD, and adding about 10 Australian tax and finance tasks (6.2). Until the sets are scored, GLM-5.3-Flash carries those seats unproven (6.2).</t>
         </is>
       </c>
       <c r="D24" s="16" t="n"/>
@@ -9546,7 +9546,7 @@
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>Open, after Day 1 (v0.4.0; the 40-task design and its promotion rule approved on 2026-10-17, S56): write 8 to 10 one-paragraph real situations that would warrant TF_OMEGA, from which ATLAS drafts the trial's apex tasks; approve the 40 drafted tasks and references, the planted flaws included; grade the split verdicts and 10 calibration tasks blind (D-46 option (b), T-30; to-do trial-task-set).</t>
+          <t>Open, for the live ATLAS (S57): the list of Australian Standards you hold or subscribe to, with each licence's terms checked: whether it allows storing and processing the text in a private system. ATLAS holds the text of only those; every other standard it cites by number, edition and what free sources say, never its clauses (8.4). Accepting or renewing a licence stays your own act (16.3 item 2). Until the list is given, no standard's text is held. It also serves the D-49 test sets (to-do seat-test-sets).</t>
         </is>
       </c>
       <c r="D25" s="16" t="n"/>
@@ -9563,7 +9563,7 @@
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Open, after Day 1 (S56, D-19 (c)): supply 20 to 30 of your own coding tasks for T-03. They run on GLM-5.3-Flash and DeepSeek-V4-Flash-0731 at each seat's real settings, and the result decides which of the two codes (17). Until then GLM-5.3-Flash codes.</t>
+          <t>Open, after Day 1 (v0.4.0; the 40-task design and its promotion rule approved on 2026-10-17, S56): write 8 to 10 one-paragraph real situations that would warrant TF_OMEGA, from which ATLAS drafts the trial's apex tasks; approve the 40 drafted tasks and references, the planted flaws included; grade the split verdicts and 10 calibration tasks blind (D-46 option (b), T-30; to-do trial-task-set).</t>
         </is>
       </c>
       <c r="D26" s="16" t="n"/>
@@ -9580,7 +9580,7 @@
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>Optional, asked at the prompt (v0.3.1, relaxed in v0.3.3): have the Cloudflare zone id for sovereign-node.link to hand (Overview page of the zone). A Zone:DNS:Edit-only token cannot look the zone up by name; Phase 1 step 7 asks for the id once if the token cannot list zones. A missing CLOUDFLARE.txt or a skipped zone id defers dynamic DNS and V23 with a to-do.</t>
+          <t>Open, after Day 1 (S56, D-19 (c)): supply 20 to 30 of your own coding tasks for T-03. They run on GLM-5.3-Flash and DeepSeek-V4-Flash-0731 at each seat's real settings, and the result decides which of the two codes (17). Until then GLM-5.3-Flash codes.</t>
         </is>
       </c>
       <c r="D27" s="16" t="n"/>
@@ -9597,14 +9597,10 @@
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>Source reference recordings for Alaric's gravelly voice and, if the British male presets collide, Gideon's. Sourced. Drop them as alaric.* and gideon.* (WAV, MP3 or M4A; step 5 converts to 16 kHz mono WAV) into /srv/atlas/staging/inbox/voice-references/ once Phase 1 has created the folder; if absent, both fall back to the nearest Kokoro preset and V7 is recorded as deferred, not failed.</t>
-        </is>
-      </c>
-      <c r="D28" s="16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>Optional, asked at the prompt (v0.3.1, relaxed in v0.3.3): have the Cloudflare zone id for sovereign-node.link to hand (Overview page of the zone). A Zone:DNS:Edit-only token cannot look the zone up by name; Phase 1 step 7 asks for the id once if the token cannot list zones. A missing CLOUDFLARE.txt or a skipped zone id defers dynamic DNS and V23 with a to-do.</t>
+        </is>
+      </c>
+      <c r="D28" s="16" t="n"/>
       <c r="E28" s="17" t="n"/>
     </row>
     <row r="29">
@@ -9618,7 +9614,7 @@
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>Have a monitor and keyboard available for Phase 1 only, in case first boot needs a hand. Done.</t>
+          <t>Source reference recordings for Alaric's gravelly voice and, if the British male presets collide, Gideon's. Sourced. Drop them as alaric.* and gideon.* (WAV, MP3 or M4A; step 5 converts to 16 kHz mono WAV) into /srv/atlas/staging/inbox/voice-references/ once Phase 1 has created the folder; if absent, both fall back to the nearest Kokoro preset and V7 is recorded as deferred, not failed.</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
@@ -9634,12 +9630,12 @@
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>Automated on the Principal's instruction, no action needed</t>
+          <t>Principal's actions — what is genuinely left</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>Cloudflare token relocation and deletion of CLOUDFLARE.txt: Phase 2 step 6b (V23).</t>
+          <t>Have a monitor and keyboard available for Phase 1 only, in case first boot needs a hand. Done.</t>
         </is>
       </c>
       <c r="D30" s="16" t="inlineStr">
@@ -9660,7 +9656,7 @@
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>Director aliases generated from names rather than confirmed one by one (D14).</t>
+          <t>Cloudflare token relocation and deletion of CLOUDFLARE.txt: Phase 2 step 6b (V23).</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
@@ -9676,12 +9672,12 @@
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>Build-side preconditions</t>
+          <t>Automated on the Principal's instruction, no action needed</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Ubuntu Server 26.04.1 installed on the 4 TB drive with the installer's encrypted-LVM (LUKS) option (installer storage step: *Use an entire disk*, the 4 TB drive, tick *Encrypt the LVM group with LUKS*, choose a disk passphrase; Section 3.5 requires both volumes encrypted; v0.3.3: an unencrypted OS volume is a warning and the to-do os-volume-encryption, not a stop); 8 TB drive unpartitioned. No desktop needed at install time: Phase 1 step 5b installs XFCE, xrdp and Chrome. Done per the returned workbook; confirm the encryption option was taken.</t>
+          <t>Director aliases generated from names rather than confirmed one by one (D14).</t>
         </is>
       </c>
       <c r="D32" s="16" t="inlineStr">
@@ -9702,7 +9698,7 @@
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>BIOS: UMA minimum, IOMMU on, fTPM on. Done. Secure Boot: enabled (D15, v0.3.3; see the Principal's actions above).</t>
+          <t>Ubuntu Server 26.04.1 installed on the 4 TB drive with the installer's encrypted-LVM (LUKS) option (installer storage step: *Use an entire disk*, the 4 TB drive, tick *Encrypt the LVM group with LUKS*, choose a disk passphrase; Section 3.5 requires both volumes encrypted; v0.3.3: an unencrypted OS volume is a warning and the to-do os-volume-encryption, not a stop); 8 TB drive unpartitioned. No desktop needed at install time: Phase 1 step 5b installs XFCE, xrdp and Chrome. Done per the returned workbook; confirm the encryption option was taken.</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
@@ -9723,7 +9719,7 @@
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>LAN address reserved for the node on the router (DHCP reservation for the node's MAC, Wi-Fi or cable: Phase 1 uses whichever interface is up); UDP 51820 forward confirmed to that address. Done. The reservation is what keeps the forward pointing at the node; no further IP action is needed beyond that move, and the VPN test from mobile data (V5) can be done whenever convenient. *S56:* the reservation and the forward move to the cable port's MAC before Phase 1 (box below).</t>
+          <t>BIOS: UMA minimum, IOMMU on, fTPM on. Done. Secure Boot: enabled (D15, v0.3.3; see the Principal's actions above).</t>
         </is>
       </c>
       <c r="D34" s="16" t="inlineStr">
@@ -9744,10 +9740,14 @@
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>New in S56 (B-27, the Principal's choice of 2026-10-17), before Phase 1: plug the cable into the node's 10 GbE port not marked DASH (the one away from DC IN) and into a 2.5 GbE router port; move the DHCP reservation and the UDP 51820 forward above to that port's MAC; take Wi-Fi off the LAN subnet. Pre-flight notes the port and the MAC and warns, never stops, if any of this is missing. A move after Phase 1 means setting LAN_IFACE and LAN_CIDR and re-running Phase 1 step 4 (--force 04).</t>
-        </is>
-      </c>
-      <c r="D35" s="16" t="n"/>
+          <t>LAN address reserved for the node on the router (DHCP reservation for the node's MAC, Wi-Fi or cable: Phase 1 uses whichever interface is up); UDP 51820 forward confirmed to that address. Done. The reservation is what keeps the forward pointing at the node; no further IP action is needed beyond that move, and the VPN test from mobile data (V5) can be done whenever convenient. *S56:* the reservation and the forward move to the cable port's MAC before Phase 1 (box below).</t>
+        </is>
+      </c>
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="E35" s="17" t="n"/>
     </row>
     <row r="36">
@@ -9761,14 +9761,10 @@
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>Internet bandwidth known, so the Phase 3 download can be planned (v0.4.0: about 448 GB in Phase 3, about 10 hours at 100 Mbps, D-42 option (b); about 842 GB of phased engines later; about 1.9 TB in all, D-41 option (a); v0.3.5 planned ~690 GB). Done; recorded on 2026-10-17 (S56, B-27): a 2,000 Mbps line, with 400 Mbps planned for the single-stream pull as written: about 2.5 hours for Phase 3's 448 GB, about 4.2 hours for the 757 GB of phased engines and about 10 hours for about 1.8 TB in all (15.4).</t>
-        </is>
-      </c>
-      <c r="D36" s="16" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>New in S56 (B-27, the Principal's choice of 2026-10-17), before Phase 1: plug the cable into the node's 10 GbE port not marked DASH (the one away from DC IN) and into a 2.5 GbE router port; move the DHCP reservation and the UDP 51820 forward above to that port's MAC; take Wi-Fi off the LAN subnet. Pre-flight notes the port and the MAC and warns, never stops, if any of this is missing. A move after Phase 1 means setting LAN_IFACE and LAN_CIDR and re-running Phase 1 step 4 (--force 04).</t>
+        </is>
+      </c>
+      <c r="D36" s="16" t="n"/>
       <c r="E36" s="17" t="n"/>
     </row>
     <row r="37">
@@ -9777,12 +9773,12 @@
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>Accepted resolutions</t>
+          <t>Build-side preconditions</t>
         </is>
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>C1 through C20 accepted in the returned workbook. C19 was reopened and re-decided in the Principal's favour.</t>
+          <t>Internet bandwidth known, so the Phase 3 download can be planned (v0.4.0: about 448 GB in Phase 3, about 10 hours at 100 Mbps, D-42 option (b); about 842 GB of phased engines later; about 1.9 TB in all, D-41 option (a); v0.3.5 planned ~690 GB). Done; recorded on 2026-10-17 (S56, B-27): a 2,000 Mbps line, with 400 Mbps planned for the single-stream pull as written: about 2.5 hours for Phase 3's 448 GB, about 4.2 hours for the 757 GB of phased engines and about 10 hours for about 1.8 TB in all (15.4).</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
@@ -9803,7 +9799,7 @@
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>C21 through C26, new in v0.2, accepted in the returned workbook: the Ubuntu and amd64v3 rejections, the quantisation rise, the closed reserve list, the vision consolidation, and the residency-versus-generation reading.</t>
+          <t>C1 through C20 accepted in the returned workbook. C19 was reopened and re-decided in the Principal's favour.</t>
         </is>
       </c>
       <c r="D38" s="16" t="inlineStr">
@@ -9824,7 +9820,7 @@
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>R9, R16, R19, R20 and R21 acknowledged in the returned workbook: two changed wording in v0.2, three were new.</t>
+          <t>C21 through C26, new in v0.2, accepted in the returned workbook: the Ubuntu and amd64v3 rejections, the quantisation rise, the closed reserve list, the vision consolidation, and the residency-versus-generation reading.</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
@@ -9845,7 +9841,7 @@
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>C27, new in v0.3.4: Ubuntu Server 26.04.1 kept over Fedora 44 KDE Plasma. Decided by the Principal on 2026-10-08.</t>
+          <t>R9, R16, R19, R20 and R21 acknowledged in the returned workbook: two changed wording in v0.2, three were new.</t>
         </is>
       </c>
       <c r="D40" s="16" t="inlineStr">
@@ -9866,7 +9862,7 @@
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>R22 to R25 acknowledged by the Principal on 2026-10-08 (R22 and R23 new in v0.3.2, R24 and R25 new in v0.3.4).</t>
+          <t>C27, new in v0.3.4: Ubuntu Server 26.04.1 kept over Fedora 44 KDE Plasma. Decided by the Principal on 2026-10-08.</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
@@ -9887,7 +9883,7 @@
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>R26 to R28 acknowledged by the Principal on 2026-10-13 (all three new in v0.3.5, S53, 2026-10-12; sheet 3).</t>
+          <t>R22 to R25 acknowledged by the Principal on 2026-10-08 (R22 and R23 new in v0.3.2, R24 and R25 new in v0.3.4).</t>
         </is>
       </c>
       <c r="D42" s="16" t="inlineStr">
@@ -9908,7 +9904,7 @@
       </c>
       <c r="C43" s="11" t="inlineStr">
         <is>
-          <t>C28 to C30, new in v0.4.0 (superseding C23, C25 and C26), and D16 to D27 (reopening D4, D10 and D12): approved by the Principal on 2026-10-16 in the returned action register (D-25 option (a)).</t>
+          <t>R26 to R28 acknowledged by the Principal on 2026-10-13 (all three new in v0.3.5, S53, 2026-10-12; sheet 3).</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
@@ -9929,7 +9925,7 @@
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>R29 to R33 and the restated R4, R17, R19 and R20 acknowledged by the Principal on 2026-10-17 (R29 to R33 new in v0.4.0, S-47, 2026-10-16; the four restated in S-47 and S-48; S55; sheet 3).</t>
+          <t>C28 to C30, new in v0.4.0 (superseding C23, C25 and C26), and D16 to D27 (reopening D4, D10 and D12): approved by the Principal on 2026-10-16 in the returned action register (D-25 option (a)).</t>
         </is>
       </c>
       <c r="D44" s="16" t="inlineStr">
@@ -9950,19 +9946,40 @@
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
+          <t>R29 to R33 and the restated R4, R17, R19 and R20 acknowledged by the Principal on 2026-10-17 (R29 to R33 new in v0.4.0, S-47, 2026-10-16; the four restated in S-47 and S-48; S55; sheet 3).</t>
+        </is>
+      </c>
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E45" s="17" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="12" t="n">
+        <v>42</v>
+      </c>
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>Accepted resolutions</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="inlineStr">
+        <is>
           <t>R9 and R20 restated in S56 with B-27 (R9 applicable with the cable; R20 lowered to Low), and R33's mitigation naming the node's own sampling settings (D-47): approved by the Principal on 2026-10-17 with those recommendations (sheet 3).</t>
         </is>
       </c>
-      <c r="D45" s="16" t="inlineStr">
+      <c r="D46" s="16" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E45" s="17" t="n"/>
+      <c r="E46" s="17" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E45"/>
-  <conditionalFormatting sqref="D5:D45">
+  <autoFilter ref="A4:E46"/>
+  <conditionalFormatting sqref="D5:D46">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Yes"</formula>
     </cfRule>
@@ -9974,7 +9991,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="D5:D45" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Choose" prompt="Pick one: Yes / No / N/A" type="list" errorStyle="stop">
+    <dataValidation sqref="D5:D46" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list." promptTitle="Choose" prompt="Pick one: Yes / No / N/A" type="list" errorStyle="stop">
       <formula1>"Yes,No,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10995,7 +11012,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Section 8.2. Thirty original domains retained and six added, thirty-six in all. Tier A loads freely, B on clear match, C on explicit match only.</t>
+          <t>Section 8.2. Thirty original domains retained and six added, thirty-six in all. Tier A loads freely, B on clear match, C on explicit match only. S57 (2026-10-17): a compliance list's Australian law is that of the Commonwealth, VIC, NSW and QLD, the Principal's main locations; Australian Standards are cited by number unless the Principal holds a licence for the text (8.4).</t>
         </is>
       </c>
     </row>

</xml_diff>